<commit_message>
Refactored code to include data classes to expose properties and provide get and set methods. This will improve code readability, maintainability, and scalability.
Completed: EquipmentData, StockpileData, GradeBlockData
Remaining: CrusherData, EventPool
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/output/build_report_2024-11-28_06-00.xlsx
+++ b/blendmaster_backend_OOP/output/build_report_2024-11-28_06-00.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L608"/>
+  <dimension ref="A1:L607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20586,32 +20586,32 @@
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0106</t>
+          <t>CEN01_RP01_0107</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>171.5431458111511</v>
+        <v>240</v>
       </c>
       <c r="F504" s="2" t="n">
-        <v>45625.56427019872</v>
+        <v>45625.56376538513</v>
       </c>
       <c r="G504" t="n">
-        <v>445744.7353634185</v>
+        <v>372370.9866868142</v>
       </c>
       <c r="H504" t="n">
-        <v>60.88547961380101</v>
+        <v>59.52524598312571</v>
       </c>
       <c r="I504" t="n">
-        <v>3.876761165120385</v>
+        <v>4.135327298523092</v>
       </c>
       <c r="J504" t="n">
-        <v>2.516358845756266</v>
+        <v>3.32028289040059</v>
       </c>
       <c r="K504" t="n">
-        <v>0.114023005291366</v>
+        <v>0.1407428129768286</v>
       </c>
       <c r="L504" t="n">
-        <v>0.041376618923828</v>
+        <v>0.04837176857847136</v>
       </c>
     </row>
     <row r="505">
@@ -20633,25 +20633,25 @@
         <v>240</v>
       </c>
       <c r="F505" s="2" t="n">
-        <v>45625.56376538513</v>
+        <v>45625.25234285779</v>
       </c>
       <c r="G505" t="n">
-        <v>372370.9866868142</v>
+        <v>372610.9866868142</v>
       </c>
       <c r="H505" t="n">
-        <v>59.52524598312571</v>
+        <v>59.52598767269989</v>
       </c>
       <c r="I505" t="n">
-        <v>4.135327298523092</v>
+        <v>4.13477551685537</v>
       </c>
       <c r="J505" t="n">
-        <v>3.32028289040059</v>
+        <v>3.320874886541835</v>
       </c>
       <c r="K505" t="n">
-        <v>0.1407428129768286</v>
+        <v>0.140740873701981</v>
       </c>
       <c r="L505" t="n">
-        <v>0.04837176857847136</v>
+        <v>0.04836762327810713</v>
       </c>
     </row>
     <row r="506">
@@ -20673,25 +20673,25 @@
         <v>240</v>
       </c>
       <c r="F506" s="2" t="n">
-        <v>45625.25234285779</v>
+        <v>45625.25723553456</v>
       </c>
       <c r="G506" t="n">
-        <v>372610.9866868142</v>
+        <v>372850.9866868142</v>
       </c>
       <c r="H506" t="n">
-        <v>59.52598767269989</v>
+        <v>59.52672840743954</v>
       </c>
       <c r="I506" t="n">
-        <v>4.13477551685537</v>
+        <v>4.134224445538995</v>
       </c>
       <c r="J506" t="n">
-        <v>3.320874886541835</v>
+        <v>3.321466120560521</v>
       </c>
       <c r="K506" t="n">
-        <v>0.140740873701981</v>
+        <v>0.1407389369237123</v>
       </c>
       <c r="L506" t="n">
-        <v>0.04836762327810713</v>
+        <v>0.04836348331430963</v>
       </c>
     </row>
     <row r="507">
@@ -20713,25 +20713,25 @@
         <v>240</v>
       </c>
       <c r="F507" s="2" t="n">
-        <v>45625.25723553456</v>
+        <v>45625.26212821133</v>
       </c>
       <c r="G507" t="n">
-        <v>372850.9866868142</v>
+        <v>373090.9866868142</v>
       </c>
       <c r="H507" t="n">
-        <v>59.52672840743954</v>
+        <v>59.52746818918732</v>
       </c>
       <c r="I507" t="n">
-        <v>4.134224445538995</v>
+        <v>4.133674083203113</v>
       </c>
       <c r="J507" t="n">
-        <v>3.321466120560521</v>
+        <v>3.322056593927412</v>
       </c>
       <c r="K507" t="n">
-        <v>0.1407389369237123</v>
+        <v>0.1407370026372046</v>
       </c>
       <c r="L507" t="n">
-        <v>0.04836348331430963</v>
+        <v>0.04835934867678023</v>
       </c>
     </row>
     <row r="508">
@@ -20753,25 +20753,25 @@
         <v>240</v>
       </c>
       <c r="F508" s="2" t="n">
-        <v>45625.26212821133</v>
+        <v>45625.2670208881</v>
       </c>
       <c r="G508" t="n">
-        <v>373090.9866868142</v>
+        <v>373330.9866868142</v>
       </c>
       <c r="H508" t="n">
-        <v>59.52746818918732</v>
+        <v>59.52820701978117</v>
       </c>
       <c r="I508" t="n">
-        <v>4.133674083203113</v>
+        <v>4.133124428480397</v>
       </c>
       <c r="J508" t="n">
-        <v>3.322056593927412</v>
+        <v>3.322646308109488</v>
       </c>
       <c r="K508" t="n">
-        <v>0.1407370026372046</v>
+        <v>0.1407350708376523</v>
       </c>
       <c r="L508" t="n">
-        <v>0.04835934867678023</v>
+        <v>0.04835521935524679</v>
       </c>
     </row>
     <row r="509">
@@ -20793,25 +20793,25 @@
         <v>240</v>
       </c>
       <c r="F509" s="2" t="n">
-        <v>45625.2670208881</v>
+        <v>45625.27191356487</v>
       </c>
       <c r="G509" t="n">
-        <v>373330.9866868142</v>
+        <v>373570.9866868142</v>
       </c>
       <c r="H509" t="n">
-        <v>59.52820701978117</v>
+        <v>59.52894490105428</v>
       </c>
       <c r="I509" t="n">
-        <v>4.133124428480397</v>
+        <v>4.132575480007032</v>
       </c>
       <c r="J509" t="n">
-        <v>3.322646308109488</v>
+        <v>3.323235264569959</v>
       </c>
       <c r="K509" t="n">
-        <v>0.1407350708376523</v>
+        <v>0.1407331415202623</v>
       </c>
       <c r="L509" t="n">
-        <v>0.04835521935524679</v>
+        <v>0.04835109533946354</v>
       </c>
     </row>
     <row r="510">
@@ -20833,25 +20833,25 @@
         <v>240</v>
       </c>
       <c r="F510" s="2" t="n">
-        <v>45625.27191356487</v>
+        <v>45625.27680624164</v>
       </c>
       <c r="G510" t="n">
-        <v>373570.9866868142</v>
+        <v>373810.9866868142</v>
       </c>
       <c r="H510" t="n">
-        <v>59.52894490105428</v>
+        <v>59.52968183483515</v>
       </c>
       <c r="I510" t="n">
-        <v>4.132575480007032</v>
+        <v>4.132027236422705</v>
       </c>
       <c r="J510" t="n">
-        <v>3.323235264569959</v>
+        <v>3.323823464768279</v>
       </c>
       <c r="K510" t="n">
-        <v>0.1407331415202623</v>
+        <v>0.1407312146802535</v>
       </c>
       <c r="L510" t="n">
-        <v>0.04835109533946354</v>
+        <v>0.04834697661921106</v>
       </c>
     </row>
     <row r="511">
@@ -20873,25 +20873,25 @@
         <v>240</v>
       </c>
       <c r="F511" s="2" t="n">
-        <v>45625.27680624164</v>
+        <v>45625.28169891841</v>
       </c>
       <c r="G511" t="n">
-        <v>373810.9866868142</v>
+        <v>374050.9866868142</v>
       </c>
       <c r="H511" t="n">
-        <v>59.52968183483515</v>
+        <v>59.53041782294756</v>
       </c>
       <c r="I511" t="n">
-        <v>4.132027236422705</v>
+        <v>4.131479696370597</v>
       </c>
       <c r="J511" t="n">
-        <v>3.323823464768279</v>
+        <v>3.324410910160155</v>
       </c>
       <c r="K511" t="n">
-        <v>0.1407312146802535</v>
+        <v>0.1407292903128574</v>
       </c>
       <c r="L511" t="n">
-        <v>0.04834697661921106</v>
+        <v>0.0483428631842961</v>
       </c>
     </row>
     <row r="512">
@@ -20913,25 +20913,25 @@
         <v>240</v>
       </c>
       <c r="F512" s="2" t="n">
-        <v>45625.28169891841</v>
+        <v>45625.28659159518</v>
       </c>
       <c r="G512" t="n">
-        <v>374050.9866868142</v>
+        <v>374290.9866868142</v>
       </c>
       <c r="H512" t="n">
-        <v>59.53041782294756</v>
+        <v>59.53115286721066</v>
       </c>
       <c r="I512" t="n">
-        <v>4.131479696370597</v>
+        <v>4.130932858497367</v>
       </c>
       <c r="J512" t="n">
-        <v>3.324410910160155</v>
+        <v>3.32499760219756</v>
       </c>
       <c r="K512" t="n">
-        <v>0.1407292903128574</v>
+        <v>0.1407273684133175</v>
       </c>
       <c r="L512" t="n">
-        <v>0.0483428631842961</v>
+        <v>0.04833875502455161</v>
       </c>
     </row>
     <row r="513">
@@ -20953,25 +20953,25 @@
         <v>240</v>
       </c>
       <c r="F513" s="2" t="n">
-        <v>45625.28659159518</v>
+        <v>45625.29148427195</v>
       </c>
       <c r="G513" t="n">
-        <v>374290.9866868142</v>
+        <v>374530.9866868142</v>
       </c>
       <c r="H513" t="n">
-        <v>59.53115286721066</v>
+        <v>59.53188696943889</v>
       </c>
       <c r="I513" t="n">
-        <v>4.130932858497367</v>
+        <v>4.130386721453143</v>
       </c>
       <c r="J513" t="n">
-        <v>3.32499760219756</v>
+        <v>3.325583542328746</v>
       </c>
       <c r="K513" t="n">
-        <v>0.1407273684133175</v>
+        <v>0.1407254489768897</v>
       </c>
       <c r="L513" t="n">
-        <v>0.04833875502455161</v>
+        <v>0.04833465212983658</v>
       </c>
     </row>
     <row r="514">
@@ -20993,25 +20993,25 @@
         <v>240</v>
       </c>
       <c r="F514" s="2" t="n">
-        <v>45625.29148427195</v>
+        <v>45625.29637694873</v>
       </c>
       <c r="G514" t="n">
-        <v>374530.9866868142</v>
+        <v>374770.9866868142</v>
       </c>
       <c r="H514" t="n">
-        <v>59.53188696943889</v>
+        <v>59.53262013144207</v>
       </c>
       <c r="I514" t="n">
-        <v>4.130386721453143</v>
+        <v>4.129841283891511</v>
       </c>
       <c r="J514" t="n">
-        <v>3.325583542328746</v>
+        <v>3.326168731998256</v>
       </c>
       <c r="K514" t="n">
-        <v>0.1407254489768897</v>
+        <v>0.1407235319988418</v>
       </c>
       <c r="L514" t="n">
-        <v>0.04833465212983658</v>
+        <v>0.04833055449003598</v>
       </c>
     </row>
     <row r="515">
@@ -21033,25 +21033,25 @@
         <v>240</v>
       </c>
       <c r="F515" s="2" t="n">
-        <v>45625.29637694873</v>
+        <v>45625.3012696255</v>
       </c>
       <c r="G515" t="n">
-        <v>374770.9866868142</v>
+        <v>375010.9866868142</v>
       </c>
       <c r="H515" t="n">
-        <v>59.53262013144207</v>
+        <v>59.53335235502539</v>
       </c>
       <c r="I515" t="n">
-        <v>4.129841283891511</v>
+        <v>4.129296544469504</v>
       </c>
       <c r="J515" t="n">
-        <v>3.326168731998256</v>
+        <v>3.326753172646934</v>
       </c>
       <c r="K515" t="n">
-        <v>0.1407235319988418</v>
+        <v>0.1407216174744539</v>
       </c>
       <c r="L515" t="n">
-        <v>0.04833055449003598</v>
+        <v>0.04832646209506066</v>
       </c>
     </row>
     <row r="516">
@@ -21073,25 +21073,25 @@
         <v>240</v>
       </c>
       <c r="F516" s="2" t="n">
-        <v>45625.3012696255</v>
+        <v>45625.30616230227</v>
       </c>
       <c r="G516" t="n">
-        <v>375010.9866868142</v>
+        <v>375250.9866868142</v>
       </c>
       <c r="H516" t="n">
-        <v>59.53335235502539</v>
+        <v>59.53408364198939</v>
       </c>
       <c r="I516" t="n">
-        <v>4.129296544469504</v>
+        <v>4.128752501847591</v>
       </c>
       <c r="J516" t="n">
-        <v>3.326753172646934</v>
+        <v>3.327336865711938</v>
       </c>
       <c r="K516" t="n">
-        <v>0.1407216174744539</v>
+        <v>0.1407197053990182</v>
       </c>
       <c r="L516" t="n">
-        <v>0.04832646209506066</v>
+        <v>0.04832237493484729</v>
       </c>
     </row>
     <row r="517">
@@ -21113,25 +21113,25 @@
         <v>240</v>
       </c>
       <c r="F517" s="2" t="n">
-        <v>45625.30616230227</v>
+        <v>45625.31105497904</v>
       </c>
       <c r="G517" t="n">
-        <v>375250.9866868142</v>
+        <v>375490.9866868142</v>
       </c>
       <c r="H517" t="n">
-        <v>59.53408364198939</v>
+        <v>59.53481399413004</v>
       </c>
       <c r="I517" t="n">
-        <v>4.128752501847591</v>
+        <v>4.128209154689664</v>
       </c>
       <c r="J517" t="n">
-        <v>3.327336865711938</v>
+        <v>3.327919812626751</v>
       </c>
       <c r="K517" t="n">
-        <v>0.1407197053990182</v>
+        <v>0.1407177957678388</v>
       </c>
       <c r="L517" t="n">
-        <v>0.04832237493484729</v>
+        <v>0.04831829299935827</v>
       </c>
     </row>
     <row r="518">
@@ -21153,25 +21153,25 @@
         <v>240</v>
       </c>
       <c r="F518" s="2" t="n">
-        <v>45625.31105497904</v>
+        <v>45625.31594765581</v>
       </c>
       <c r="G518" t="n">
-        <v>375490.9866868142</v>
+        <v>375730.9866868142</v>
       </c>
       <c r="H518" t="n">
-        <v>59.53481399413004</v>
+        <v>59.53554341323871</v>
       </c>
       <c r="I518" t="n">
-        <v>4.128209154689664</v>
+        <v>4.127666501663031</v>
       </c>
       <c r="J518" t="n">
-        <v>3.327919812626751</v>
+        <v>3.328502014821195</v>
       </c>
       <c r="K518" t="n">
-        <v>0.1407177957678388</v>
+        <v>0.1407158885762319</v>
       </c>
       <c r="L518" t="n">
-        <v>0.04831829299935827</v>
+        <v>0.04831421627858165</v>
       </c>
     </row>
     <row r="519">
@@ -21193,25 +21193,25 @@
         <v>240</v>
       </c>
       <c r="F519" s="2" t="n">
-        <v>45625.31594765581</v>
+        <v>45625.32084033258</v>
       </c>
       <c r="G519" t="n">
-        <v>375730.9866868142</v>
+        <v>375970.9866868142</v>
       </c>
       <c r="H519" t="n">
-        <v>59.53554341323871</v>
+        <v>59.53627190110219</v>
       </c>
       <c r="I519" t="n">
-        <v>4.127666501663031</v>
+        <v>4.127124541438401</v>
       </c>
       <c r="J519" t="n">
-        <v>3.328502014821195</v>
+        <v>3.32908347372144</v>
       </c>
       <c r="K519" t="n">
-        <v>0.1407158885762319</v>
+        <v>0.1407139838195255</v>
       </c>
       <c r="L519" t="n">
-        <v>0.04831421627858165</v>
+        <v>0.04831014476253104</v>
       </c>
     </row>
     <row r="520">
@@ -21233,25 +21233,25 @@
         <v>240</v>
       </c>
       <c r="F520" s="2" t="n">
-        <v>45625.32084033258</v>
+        <v>45625.32573300935</v>
       </c>
       <c r="G520" t="n">
-        <v>375970.9866868142</v>
+        <v>376210.9866868142</v>
       </c>
       <c r="H520" t="n">
-        <v>59.53627190110219</v>
+        <v>59.53699945950272</v>
       </c>
       <c r="I520" t="n">
-        <v>4.127124541438401</v>
+        <v>4.126583272689877</v>
       </c>
       <c r="J520" t="n">
-        <v>3.32908347372144</v>
+        <v>3.329664190750017</v>
       </c>
       <c r="K520" t="n">
-        <v>0.1407139838195255</v>
+        <v>0.1407120814930597</v>
       </c>
       <c r="L520" t="n">
-        <v>0.04831014476253104</v>
+        <v>0.04830607844124554</v>
       </c>
     </row>
     <row r="521">
@@ -21273,25 +21273,25 @@
         <v>240</v>
       </c>
       <c r="F521" s="2" t="n">
-        <v>45625.32573300935</v>
+        <v>45625.33062568613</v>
       </c>
       <c r="G521" t="n">
-        <v>376210.9866868142</v>
+        <v>376450.9866868142</v>
       </c>
       <c r="H521" t="n">
-        <v>59.53699945950272</v>
+        <v>59.53772609021799</v>
       </c>
       <c r="I521" t="n">
-        <v>4.126583272689877</v>
+        <v>4.126042694094941</v>
       </c>
       <c r="J521" t="n">
-        <v>3.329664190750017</v>
+        <v>3.330244167325831</v>
       </c>
       <c r="K521" t="n">
-        <v>0.1407120814930597</v>
+        <v>0.1407101815921865</v>
       </c>
       <c r="L521" t="n">
-        <v>0.04830607844124554</v>
+        <v>0.04830201730478962</v>
       </c>
     </row>
     <row r="522">
@@ -21313,25 +21313,25 @@
         <v>240</v>
       </c>
       <c r="F522" s="2" t="n">
-        <v>45625.33062568613</v>
+        <v>45625.3355183629</v>
       </c>
       <c r="G522" t="n">
-        <v>376450.9866868142</v>
+        <v>376690.9866868142</v>
       </c>
       <c r="H522" t="n">
-        <v>59.53772609021799</v>
+        <v>59.53845179502115</v>
       </c>
       <c r="I522" t="n">
-        <v>4.126042694094941</v>
+        <v>4.125502804334446</v>
       </c>
       <c r="J522" t="n">
-        <v>3.330244167325831</v>
+        <v>3.330823404864167</v>
       </c>
       <c r="K522" t="n">
-        <v>0.1407101815921865</v>
+        <v>0.1407082841122695</v>
       </c>
       <c r="L522" t="n">
-        <v>0.04830201730478962</v>
+        <v>0.04829796134325312</v>
       </c>
     </row>
     <row r="523">
@@ -21353,25 +21353,25 @@
         <v>240</v>
       </c>
       <c r="F523" s="2" t="n">
-        <v>45625.3355183629</v>
+        <v>45625.34041103967</v>
       </c>
       <c r="G523" t="n">
-        <v>376690.9866868142</v>
+        <v>376930.9866868142</v>
       </c>
       <c r="H523" t="n">
-        <v>59.53845179502115</v>
+        <v>59.53917657568086</v>
       </c>
       <c r="I523" t="n">
-        <v>4.125502804334446</v>
+        <v>4.124963602092607</v>
       </c>
       <c r="J523" t="n">
-        <v>3.330823404864167</v>
+        <v>3.331401904776709</v>
       </c>
       <c r="K523" t="n">
-        <v>0.1407082841122695</v>
+        <v>0.1407063890486845</v>
       </c>
       <c r="L523" t="n">
-        <v>0.04829796134325312</v>
+        <v>0.04829391054675108</v>
       </c>
     </row>
     <row r="524">
@@ -21390,28 +21390,28 @@
         </is>
       </c>
       <c r="E524" t="n">
-        <v>240</v>
+        <v>166.2199859162001</v>
       </c>
       <c r="F524" s="2" t="n">
-        <v>45625.34041103967</v>
+        <v>45625.34530371644</v>
       </c>
       <c r="G524" t="n">
-        <v>376930.9866868142</v>
+        <v>377097.2066727304</v>
       </c>
       <c r="H524" t="n">
-        <v>59.53917657568086</v>
+        <v>59.53967800590596</v>
       </c>
       <c r="I524" t="n">
-        <v>4.124963602092607</v>
+        <v>4.124590561921236</v>
       </c>
       <c r="J524" t="n">
-        <v>3.331401904776709</v>
+        <v>3.331802132538701</v>
       </c>
       <c r="K524" t="n">
-        <v>0.1407063890486845</v>
+        <v>0.1407050779731925</v>
       </c>
       <c r="L524" t="n">
-        <v>0.04829391054675108</v>
+        <v>0.04829110805502524</v>
       </c>
     </row>
     <row r="525">
@@ -21430,28 +21430,28 @@
         </is>
       </c>
       <c r="E525" t="n">
-        <v>166.2199859162001</v>
+        <v>240</v>
       </c>
       <c r="F525" s="2" t="n">
-        <v>45625.34530371644</v>
+        <v>45625.42051092322</v>
       </c>
       <c r="G525" t="n">
-        <v>377097.2066727304</v>
+        <v>377337.2066727304</v>
       </c>
       <c r="H525" t="n">
-        <v>59.53967800590596</v>
+        <v>59.53922109426733</v>
       </c>
       <c r="I525" t="n">
-        <v>4.124590561921236</v>
+        <v>4.123987583018447</v>
       </c>
       <c r="J525" t="n">
-        <v>3.331802132538701</v>
+        <v>3.332695649006806</v>
       </c>
       <c r="K525" t="n">
-        <v>0.1407050779731925</v>
+        <v>0.1407423890600333</v>
       </c>
       <c r="L525" t="n">
-        <v>0.04829110805502524</v>
+        <v>0.04829592595804314</v>
       </c>
     </row>
     <row r="526">
@@ -21473,25 +21473,25 @@
         <v>240</v>
       </c>
       <c r="F526" s="2" t="n">
-        <v>45625.42051092322</v>
+        <v>45625.42540359999</v>
       </c>
       <c r="G526" t="n">
-        <v>377337.2066727304</v>
+        <v>377577.2066727304</v>
       </c>
       <c r="H526" t="n">
-        <v>59.53922109426733</v>
+        <v>59.53876476348364</v>
       </c>
       <c r="I526" t="n">
-        <v>4.123987583018447</v>
+        <v>4.123385370660535</v>
       </c>
       <c r="J526" t="n">
-        <v>3.332695649006806</v>
+        <v>3.333588029580326</v>
       </c>
       <c r="K526" t="n">
-        <v>0.1407423890600333</v>
+        <v>0.1407796527146632</v>
       </c>
       <c r="L526" t="n">
-        <v>0.04829592595804314</v>
+        <v>0.04830073773623833</v>
       </c>
     </row>
     <row r="527">
@@ -21513,25 +21513,25 @@
         <v>240</v>
       </c>
       <c r="F527" s="2" t="n">
-        <v>45625.42540359999</v>
+        <v>45625.43029627676</v>
       </c>
       <c r="G527" t="n">
-        <v>377577.2066727304</v>
+        <v>377817.2066727304</v>
       </c>
       <c r="H527" t="n">
-        <v>59.53876476348364</v>
+        <v>59.53830901244797</v>
       </c>
       <c r="I527" t="n">
-        <v>4.123385370660535</v>
+        <v>4.122783923386707</v>
       </c>
       <c r="J527" t="n">
-        <v>3.333588029580326</v>
+        <v>3.334479276423915</v>
       </c>
       <c r="K527" t="n">
-        <v>0.1407796527146632</v>
+        <v>0.1408168690274731</v>
       </c>
       <c r="L527" t="n">
-        <v>0.04830073773623833</v>
+        <v>0.04830554340128279</v>
       </c>
     </row>
     <row r="528">
@@ -21553,25 +21553,25 @@
         <v>240</v>
       </c>
       <c r="F528" s="2" t="n">
-        <v>45625.43029627676</v>
+        <v>45625.43518895353</v>
       </c>
       <c r="G528" t="n">
-        <v>377817.2066727304</v>
+        <v>378057.2066727304</v>
       </c>
       <c r="H528" t="n">
-        <v>59.53830901244797</v>
+        <v>59.53785384005619</v>
       </c>
       <c r="I528" t="n">
-        <v>4.122783923386707</v>
+        <v>4.122183239739881</v>
       </c>
       <c r="J528" t="n">
-        <v>3.334479276423915</v>
+        <v>3.335369391696733</v>
       </c>
       <c r="K528" t="n">
-        <v>0.1408168690274731</v>
+        <v>0.1408540380886241</v>
       </c>
       <c r="L528" t="n">
-        <v>0.04830554340128279</v>
+        <v>0.04831034296481886</v>
       </c>
     </row>
     <row r="529">
@@ -21593,25 +21593,25 @@
         <v>240</v>
       </c>
       <c r="F529" s="2" t="n">
-        <v>45625.43518895353</v>
+        <v>45625.4400816303</v>
       </c>
       <c r="G529" t="n">
-        <v>378057.2066727304</v>
+        <v>378297.2066727304</v>
       </c>
       <c r="H529" t="n">
-        <v>59.53785384005619</v>
+        <v>59.53739924520701</v>
       </c>
       <c r="I529" t="n">
-        <v>4.122183239739881</v>
+        <v>4.121583318266673</v>
       </c>
       <c r="J529" t="n">
-        <v>3.335369391696733</v>
+        <v>3.336258377552459</v>
       </c>
       <c r="K529" t="n">
-        <v>0.1408540380886241</v>
+        <v>0.1408911599880488</v>
       </c>
       <c r="L529" t="n">
-        <v>0.04831034296481886</v>
+        <v>0.04831513643845931</v>
       </c>
     </row>
     <row r="530">
@@ -21633,25 +21633,25 @@
         <v>240</v>
       </c>
       <c r="F530" s="2" t="n">
-        <v>45625.4400816303</v>
+        <v>45625.44497430707</v>
       </c>
       <c r="G530" t="n">
-        <v>378297.2066727304</v>
+        <v>378537.2066727304</v>
       </c>
       <c r="H530" t="n">
-        <v>59.53739924520701</v>
+        <v>59.5369452268019</v>
       </c>
       <c r="I530" t="n">
-        <v>4.121583318266673</v>
+        <v>4.120984157517383</v>
       </c>
       <c r="J530" t="n">
-        <v>3.336258377552459</v>
+        <v>3.337146236139312</v>
       </c>
       <c r="K530" t="n">
-        <v>0.1408911599880488</v>
+        <v>0.1409282348154514</v>
       </c>
       <c r="L530" t="n">
-        <v>0.04831513643845931</v>
+        <v>0.0483199238337875</v>
       </c>
     </row>
     <row r="531">
@@ -21673,25 +21673,25 @@
         <v>240</v>
       </c>
       <c r="F531" s="2" t="n">
-        <v>45625.44497430707</v>
+        <v>45625.44986698384</v>
       </c>
       <c r="G531" t="n">
-        <v>378537.2066727304</v>
+        <v>378777.2066727304</v>
       </c>
       <c r="H531" t="n">
-        <v>59.5369452268019</v>
+        <v>59.53649178374511</v>
       </c>
       <c r="I531" t="n">
-        <v>4.120984157517383</v>
+        <v>4.120385756045987</v>
       </c>
       <c r="J531" t="n">
-        <v>3.337146236139312</v>
+        <v>3.338032969600063</v>
       </c>
       <c r="K531" t="n">
-        <v>0.1409282348154514</v>
+        <v>0.1409652626603091</v>
       </c>
       <c r="L531" t="n">
-        <v>0.0483199238337875</v>
+        <v>0.04832470516235739</v>
       </c>
     </row>
     <row r="532">
@@ -21713,25 +21713,25 @@
         <v>240</v>
       </c>
       <c r="F532" s="2" t="n">
-        <v>45625.44986698384</v>
+        <v>45625.45475966061</v>
       </c>
       <c r="G532" t="n">
-        <v>378777.2066727304</v>
+        <v>379017.2066727304</v>
       </c>
       <c r="H532" t="n">
-        <v>59.53649178374511</v>
+        <v>59.53603891494371</v>
       </c>
       <c r="I532" t="n">
-        <v>4.120385756045987</v>
+        <v>4.119788112410123</v>
       </c>
       <c r="J532" t="n">
-        <v>3.338032969600063</v>
+        <v>3.33891858007206</v>
       </c>
       <c r="K532" t="n">
-        <v>0.1409652626603091</v>
+        <v>0.1410022436118721</v>
       </c>
       <c r="L532" t="n">
-        <v>0.04832470516235739</v>
+        <v>0.04832948043569373</v>
       </c>
     </row>
     <row r="533">
@@ -21753,25 +21753,25 @@
         <v>240</v>
       </c>
       <c r="F533" s="2" t="n">
-        <v>45625.45475966061</v>
+        <v>45625.45965233738</v>
       </c>
       <c r="G533" t="n">
-        <v>379017.2066727304</v>
+        <v>379257.2066727304</v>
       </c>
       <c r="H533" t="n">
-        <v>59.53603891494371</v>
+        <v>59.53558661930748</v>
       </c>
       <c r="I533" t="n">
-        <v>4.119788112410123</v>
+        <v>4.119191225171078</v>
       </c>
       <c r="J533" t="n">
-        <v>3.33891858007206</v>
+        <v>3.339803069687236</v>
       </c>
       <c r="K533" t="n">
-        <v>0.1410022436118721</v>
+        <v>0.1410391777591651</v>
       </c>
       <c r="L533" t="n">
-        <v>0.04832948043569373</v>
+        <v>0.04833424966529203</v>
       </c>
     </row>
     <row r="534">
@@ -21793,25 +21793,25 @@
         <v>240</v>
       </c>
       <c r="F534" s="2" t="n">
-        <v>45625.45965233738</v>
+        <v>45625.46454501415</v>
       </c>
       <c r="G534" t="n">
-        <v>379257.2066727304</v>
+        <v>379497.2066727304</v>
       </c>
       <c r="H534" t="n">
-        <v>59.53558661930748</v>
+        <v>59.53513489574899</v>
       </c>
       <c r="I534" t="n">
-        <v>4.119191225171078</v>
+        <v>4.118595092893782</v>
       </c>
       <c r="J534" t="n">
-        <v>3.339803069687236</v>
+        <v>3.340686440572135</v>
       </c>
       <c r="K534" t="n">
-        <v>0.1410391777591651</v>
+        <v>0.1410760651909871</v>
       </c>
       <c r="L534" t="n">
-        <v>0.04833424966529203</v>
+        <v>0.04833901286261877</v>
       </c>
     </row>
     <row r="535">
@@ -21833,25 +21833,25 @@
         <v>240</v>
       </c>
       <c r="F535" s="2" t="n">
-        <v>45625.46454501415</v>
+        <v>45625.46943769092</v>
       </c>
       <c r="G535" t="n">
-        <v>379497.2066727304</v>
+        <v>379737.2066727304</v>
       </c>
       <c r="H535" t="n">
-        <v>59.53513489574899</v>
+        <v>59.53468374318356</v>
       </c>
       <c r="I535" t="n">
-        <v>4.118595092893782</v>
+        <v>4.117999714146792</v>
       </c>
       <c r="J535" t="n">
-        <v>3.340686440572135</v>
+        <v>3.341568694847923</v>
       </c>
       <c r="K535" t="n">
-        <v>0.1410760651909871</v>
+        <v>0.1411129059959131</v>
       </c>
       <c r="L535" t="n">
-        <v>0.04833901286261877</v>
+        <v>0.04834377003911143</v>
       </c>
     </row>
     <row r="536">
@@ -21873,25 +21873,25 @@
         <v>240</v>
       </c>
       <c r="F536" s="2" t="n">
-        <v>45625.46943769092</v>
+        <v>45625.4743303677</v>
       </c>
       <c r="G536" t="n">
-        <v>379737.2066727304</v>
+        <v>379977.2066727304</v>
       </c>
       <c r="H536" t="n">
-        <v>59.53468374318356</v>
+        <v>59.53423316052923</v>
       </c>
       <c r="I536" t="n">
-        <v>4.117999714146792</v>
+        <v>4.117405087502278</v>
       </c>
       <c r="J536" t="n">
-        <v>3.341568694847923</v>
+        <v>3.342449834630407</v>
       </c>
       <c r="K536" t="n">
-        <v>0.1411129059959131</v>
+        <v>0.141149700262294</v>
       </c>
       <c r="L536" t="n">
-        <v>0.04834377003911143</v>
+        <v>0.04834852120617859</v>
       </c>
     </row>
     <row r="537">
@@ -21913,25 +21913,25 @@
         <v>240</v>
       </c>
       <c r="F537" s="2" t="n">
-        <v>45625.4743303677</v>
+        <v>45625.47922304447</v>
       </c>
       <c r="G537" t="n">
-        <v>379977.2066727304</v>
+        <v>380217.2066727304</v>
       </c>
       <c r="H537" t="n">
-        <v>59.53423316052923</v>
+        <v>59.53378314670681</v>
       </c>
       <c r="I537" t="n">
-        <v>4.117405087502278</v>
+        <v>4.116811211536021</v>
       </c>
       <c r="J537" t="n">
-        <v>3.342449834630407</v>
+        <v>3.343329862030053</v>
       </c>
       <c r="K537" t="n">
-        <v>0.141149700262294</v>
+        <v>0.1411864480782577</v>
       </c>
       <c r="L537" t="n">
-        <v>0.04834852120617859</v>
+        <v>0.04835326637520001</v>
       </c>
     </row>
     <row r="538">
@@ -21953,25 +21953,25 @@
         <v>240</v>
       </c>
       <c r="F538" s="2" t="n">
-        <v>45625.47922304447</v>
+        <v>45625.48411572124</v>
       </c>
       <c r="G538" t="n">
-        <v>380217.2066727304</v>
+        <v>380457.2066727304</v>
       </c>
       <c r="H538" t="n">
-        <v>59.53378314670681</v>
+        <v>59.53333370063979</v>
       </c>
       <c r="I538" t="n">
-        <v>4.116811211536021</v>
+        <v>4.11621808482739</v>
       </c>
       <c r="J538" t="n">
-        <v>3.343329862030053</v>
+        <v>3.344208779152</v>
       </c>
       <c r="K538" t="n">
-        <v>0.1411864480782577</v>
+        <v>0.1412231495317098</v>
       </c>
       <c r="L538" t="n">
-        <v>0.04835326637520001</v>
+        <v>0.04835800555752677</v>
       </c>
     </row>
     <row r="539">
@@ -21993,25 +21993,25 @@
         <v>240</v>
       </c>
       <c r="F539" s="2" t="n">
-        <v>45625.48411572124</v>
+        <v>45625.48900839801</v>
       </c>
       <c r="G539" t="n">
-        <v>380457.2066727304</v>
+        <v>380697.2066727304</v>
       </c>
       <c r="H539" t="n">
-        <v>59.53333370063979</v>
+        <v>59.53288482125438</v>
       </c>
       <c r="I539" t="n">
-        <v>4.11621808482739</v>
+        <v>4.11562570595934</v>
       </c>
       <c r="J539" t="n">
-        <v>3.344208779152</v>
+        <v>3.345086588096081</v>
       </c>
       <c r="K539" t="n">
-        <v>0.1412231495317098</v>
+        <v>0.1412598047103342</v>
       </c>
       <c r="L539" t="n">
-        <v>0.04835800555752677</v>
+        <v>0.0483627387644813</v>
       </c>
     </row>
     <row r="540">
@@ -22033,25 +22033,25 @@
         <v>240</v>
       </c>
       <c r="F540" s="2" t="n">
-        <v>45625.48900839801</v>
+        <v>45625.49390107478</v>
       </c>
       <c r="G540" t="n">
-        <v>380697.2066727304</v>
+        <v>380937.2066727304</v>
       </c>
       <c r="H540" t="n">
-        <v>59.53288482125438</v>
+        <v>59.53243650747955</v>
       </c>
       <c r="I540" t="n">
-        <v>4.11562570595934</v>
+        <v>4.115034073518395</v>
       </c>
       <c r="J540" t="n">
-        <v>3.345086588096081</v>
+        <v>3.345963290956833</v>
       </c>
       <c r="K540" t="n">
-        <v>0.1412598047103342</v>
+        <v>0.1412964137015938</v>
       </c>
       <c r="L540" t="n">
-        <v>0.0483627387644813</v>
+        <v>0.0483674660073575</v>
       </c>
     </row>
     <row r="541">
@@ -22073,25 +22073,25 @@
         <v>240</v>
       </c>
       <c r="F541" s="2" t="n">
-        <v>45625.49390107478</v>
+        <v>45625.49879375155</v>
       </c>
       <c r="G541" t="n">
-        <v>380937.2066727304</v>
+        <v>381177.2066727304</v>
       </c>
       <c r="H541" t="n">
-        <v>59.53243650747955</v>
+        <v>59.53198875824688</v>
       </c>
       <c r="I541" t="n">
-        <v>4.115034073518395</v>
+        <v>4.114443186094642</v>
       </c>
       <c r="J541" t="n">
-        <v>3.345963290956833</v>
+        <v>3.346838889823522</v>
       </c>
       <c r="K541" t="n">
-        <v>0.1412964137015938</v>
+        <v>0.1413329765927312</v>
       </c>
       <c r="L541" t="n">
-        <v>0.0483674660073575</v>
+        <v>0.04837218729742084</v>
       </c>
     </row>
     <row r="542">
@@ -22113,25 +22113,25 @@
         <v>240</v>
       </c>
       <c r="F542" s="2" t="n">
-        <v>45625.49879375155</v>
+        <v>45625.50368642832</v>
       </c>
       <c r="G542" t="n">
-        <v>381177.2066727304</v>
+        <v>381417.2066727304</v>
       </c>
       <c r="H542" t="n">
-        <v>59.53198875824688</v>
+        <v>59.53155070319304</v>
       </c>
       <c r="I542" t="n">
-        <v>4.114443186094642</v>
+        <v>4.113848104177349</v>
       </c>
       <c r="J542" t="n">
-        <v>3.346838889823522</v>
+        <v>3.347710282186754</v>
       </c>
       <c r="K542" t="n">
-        <v>0.1413329765927312</v>
+        <v>0.1413695023654911</v>
       </c>
       <c r="L542" t="n">
-        <v>0.04837218729742084</v>
+        <v>0.04837677457971879</v>
       </c>
     </row>
     <row r="543">
@@ -22153,25 +22153,25 @@
         <v>240</v>
       </c>
       <c r="F543" s="2" t="n">
-        <v>45625.50368642832</v>
+        <v>45625.51530954447</v>
       </c>
       <c r="G543" t="n">
-        <v>381417.2066727304</v>
+        <v>381657.2066727304</v>
       </c>
       <c r="H543" t="n">
-        <v>59.53155070319304</v>
+        <v>59.53194260437719</v>
       </c>
       <c r="I543" t="n">
-        <v>4.113848104177349</v>
+        <v>4.112805208253878</v>
       </c>
       <c r="J543" t="n">
-        <v>3.347710282186754</v>
+        <v>3.348298566773943</v>
       </c>
       <c r="K543" t="n">
-        <v>0.1413695023654911</v>
+        <v>0.1414067901703156</v>
       </c>
       <c r="L543" t="n">
-        <v>0.04837677457971879</v>
+        <v>0.0483697229484327</v>
       </c>
     </row>
     <row r="544">
@@ -22193,25 +22193,25 @@
         <v>240</v>
       </c>
       <c r="F544" s="2" t="n">
-        <v>45625.51530954447</v>
+        <v>45625.52020222124</v>
       </c>
       <c r="G544" t="n">
-        <v>381657.2066727304</v>
+        <v>381897.2066727304</v>
       </c>
       <c r="H544" t="n">
-        <v>59.53194260437719</v>
+        <v>59.53233401298752</v>
       </c>
       <c r="I544" t="n">
-        <v>4.112805208253878</v>
+        <v>4.111763623128272</v>
       </c>
       <c r="J544" t="n">
-        <v>3.348298566773943</v>
+        <v>3.3488861119564</v>
       </c>
       <c r="K544" t="n">
-        <v>0.1414067901703156</v>
+        <v>0.1414440311087425</v>
       </c>
       <c r="L544" t="n">
-        <v>0.0483697229484327</v>
+        <v>0.04836268018022013</v>
       </c>
     </row>
     <row r="545">
@@ -22233,25 +22233,25 @@
         <v>240</v>
       </c>
       <c r="F545" s="2" t="n">
-        <v>45625.52020222124</v>
+        <v>45625.52509489801</v>
       </c>
       <c r="G545" t="n">
-        <v>381897.2066727304</v>
+        <v>382137.2066727304</v>
       </c>
       <c r="H545" t="n">
-        <v>59.53233401298752</v>
+        <v>59.5327249299521</v>
       </c>
       <c r="I545" t="n">
-        <v>4.111763623128272</v>
+        <v>4.110723346330805</v>
       </c>
       <c r="J545" t="n">
-        <v>3.3488861119564</v>
+        <v>3.349472919127266</v>
       </c>
       <c r="K545" t="n">
-        <v>0.1414440311087425</v>
+        <v>0.1414812252690748</v>
       </c>
       <c r="L545" t="n">
-        <v>0.04836268018022013</v>
+        <v>0.0483556462583818</v>
       </c>
     </row>
     <row r="546">
@@ -22273,25 +22273,25 @@
         <v>240</v>
       </c>
       <c r="F546" s="2" t="n">
-        <v>45625.52509489801</v>
+        <v>45625.52998757478</v>
       </c>
       <c r="G546" t="n">
-        <v>382137.2066727304</v>
+        <v>382377.2066727304</v>
       </c>
       <c r="H546" t="n">
-        <v>59.5327249299521</v>
+        <v>59.53311535619667</v>
       </c>
       <c r="I546" t="n">
-        <v>4.110723346330805</v>
+        <v>4.10968437539795</v>
       </c>
       <c r="J546" t="n">
-        <v>3.349472919127266</v>
+        <v>3.350058989676187</v>
       </c>
       <c r="K546" t="n">
-        <v>0.1414812252690748</v>
+        <v>0.1415183727393935</v>
       </c>
       <c r="L546" t="n">
-        <v>0.0483556462583818</v>
+        <v>0.04834862116626037</v>
       </c>
     </row>
     <row r="547">
@@ -22313,25 +22313,25 @@
         <v>240</v>
       </c>
       <c r="F547" s="2" t="n">
-        <v>45625.52998757478</v>
+        <v>45625.53488025155</v>
       </c>
       <c r="G547" t="n">
-        <v>382377.2066727304</v>
+        <v>382617.2066727304</v>
       </c>
       <c r="H547" t="n">
-        <v>59.53311535619667</v>
+        <v>59.53350529264468</v>
       </c>
       <c r="I547" t="n">
-        <v>4.10968437539795</v>
+        <v>4.108646707872362</v>
       </c>
       <c r="J547" t="n">
-        <v>3.350058989676187</v>
+        <v>3.350644324989319</v>
       </c>
       <c r="K547" t="n">
-        <v>0.1415183727393935</v>
+        <v>0.1415554736075588</v>
       </c>
       <c r="L547" t="n">
-        <v>0.04834862116626037</v>
+        <v>0.04834160488724027</v>
       </c>
     </row>
     <row r="548">
@@ -22353,25 +22353,25 @@
         <v>240</v>
       </c>
       <c r="F548" s="2" t="n">
-        <v>45625.53488025155</v>
+        <v>45625.53977292832</v>
       </c>
       <c r="G548" t="n">
-        <v>382617.2066727304</v>
+        <v>382857.2066727304</v>
       </c>
       <c r="H548" t="n">
-        <v>59.53350529264468</v>
+        <v>59.53389474021721</v>
       </c>
       <c r="I548" t="n">
-        <v>4.108646707872362</v>
+        <v>4.107610341302857</v>
       </c>
       <c r="J548" t="n">
-        <v>3.350644324989319</v>
+        <v>3.351228926449346</v>
       </c>
       <c r="K548" t="n">
-        <v>0.1415554736075588</v>
+        <v>0.1415925279612106</v>
       </c>
       <c r="L548" t="n">
-        <v>0.04834160488724027</v>
+        <v>0.04833459740474764</v>
       </c>
     </row>
     <row r="549">
@@ -22393,25 +22393,25 @@
         <v>240</v>
       </c>
       <c r="F549" s="2" t="n">
-        <v>45625.53977292832</v>
+        <v>45625.54466560509</v>
       </c>
       <c r="G549" t="n">
-        <v>382857.2066727304</v>
+        <v>383097.2066727304</v>
       </c>
       <c r="H549" t="n">
-        <v>59.53389474021721</v>
+        <v>59.53428369983309</v>
       </c>
       <c r="I549" t="n">
-        <v>4.107610341302857</v>
+        <v>4.106575273244396</v>
       </c>
       <c r="J549" t="n">
-        <v>3.351228926449346</v>
+        <v>3.351812795435483</v>
       </c>
       <c r="K549" t="n">
-        <v>0.1415925279612106</v>
+        <v>0.1416295358877691</v>
       </c>
       <c r="L549" t="n">
-        <v>0.04833459740474764</v>
+        <v>0.0483275987022501</v>
       </c>
     </row>
     <row r="550">
@@ -22433,25 +22433,25 @@
         <v>240</v>
       </c>
       <c r="F550" s="2" t="n">
-        <v>45625.54466560509</v>
+        <v>45625.54955828186</v>
       </c>
       <c r="G550" t="n">
-        <v>383097.2066727304</v>
+        <v>383337.2066727304</v>
       </c>
       <c r="H550" t="n">
-        <v>59.53428369983309</v>
+        <v>59.5346721724088</v>
       </c>
       <c r="I550" t="n">
-        <v>4.106575273244396</v>
+        <v>4.10554150125806</v>
       </c>
       <c r="J550" t="n">
-        <v>3.351812795435483</v>
+        <v>3.352395933323495</v>
       </c>
       <c r="K550" t="n">
-        <v>0.1416295358877691</v>
+        <v>0.1416664974744356</v>
       </c>
       <c r="L550" t="n">
-        <v>0.0483275987022501</v>
+        <v>0.0483206087632567</v>
       </c>
     </row>
     <row r="551">
@@ -22473,25 +22473,25 @@
         <v>240</v>
       </c>
       <c r="F551" s="2" t="n">
-        <v>45625.54955828186</v>
+        <v>45625.55445095863</v>
       </c>
       <c r="G551" t="n">
-        <v>383337.2066727304</v>
+        <v>383577.2066727304</v>
       </c>
       <c r="H551" t="n">
-        <v>59.5346721724088</v>
+        <v>59.53506015885856</v>
       </c>
       <c r="I551" t="n">
-        <v>4.10554150125806</v>
+        <v>4.104509022911035</v>
       </c>
       <c r="J551" t="n">
-        <v>3.352395933323495</v>
+        <v>3.352978341485701</v>
       </c>
       <c r="K551" t="n">
-        <v>0.1416664974744356</v>
+        <v>0.1417034128081932</v>
       </c>
       <c r="L551" t="n">
-        <v>0.0483206087632567</v>
+        <v>0.04831362757131777</v>
       </c>
     </row>
     <row r="552">
@@ -22513,25 +22513,25 @@
         <v>240</v>
       </c>
       <c r="F552" s="2" t="n">
-        <v>45625.55445095863</v>
+        <v>45625.5593436354</v>
       </c>
       <c r="G552" t="n">
-        <v>383577.2066727304</v>
+        <v>383817.2066727304</v>
       </c>
       <c r="H552" t="n">
-        <v>59.53506015885856</v>
+        <v>59.53544766009427</v>
       </c>
       <c r="I552" t="n">
-        <v>4.104509022911035</v>
+        <v>4.103477835776593</v>
       </c>
       <c r="J552" t="n">
-        <v>3.352978341485701</v>
+        <v>3.353560021290989</v>
       </c>
       <c r="K552" t="n">
-        <v>0.1417034128081932</v>
+        <v>0.1417402819758075</v>
       </c>
       <c r="L552" t="n">
-        <v>0.04831362757131777</v>
+        <v>0.04830665511002476</v>
       </c>
     </row>
     <row r="553">
@@ -22553,65 +22553,65 @@
         <v>240</v>
       </c>
       <c r="F553" s="2" t="n">
-        <v>45625.5593436354</v>
+        <v>45625.56423631217</v>
       </c>
       <c r="G553" t="n">
-        <v>383817.2066727304</v>
+        <v>384057.2066727304</v>
       </c>
       <c r="H553" t="n">
-        <v>59.53544766009427</v>
+        <v>59.5358346770256</v>
       </c>
       <c r="I553" t="n">
-        <v>4.103477835776593</v>
+        <v>4.10244793743407</v>
       </c>
       <c r="J553" t="n">
-        <v>3.353560021290989</v>
+        <v>3.354140974104824</v>
       </c>
       <c r="K553" t="n">
-        <v>0.1417402819758075</v>
+        <v>0.1417771050638269</v>
       </c>
       <c r="L553" t="n">
-        <v>0.04830665511002476</v>
+        <v>0.04829969136301014</v>
       </c>
     </row>
     <row r="554">
       <c r="A554" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B554" s="2" t="n">
-        <v>45625.25</v>
+        <v>45625.56427019872</v>
       </c>
       <c r="C554" s="2" t="n">
+        <v>45625.75</v>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>CEN01_RP01_0106</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>171.5431458111511</v>
+      </c>
+      <c r="F554" s="2" t="n">
         <v>45625.56427019872</v>
       </c>
-      <c r="D554" t="inlineStr">
-        <is>
-          <t>CEN01_RP01_0107</t>
-        </is>
-      </c>
-      <c r="E554" t="n">
-        <v>240</v>
-      </c>
-      <c r="F554" s="2" t="n">
-        <v>45625.56423631217</v>
-      </c>
       <c r="G554" t="n">
-        <v>384057.2066727304</v>
+        <v>441287.2201325851</v>
       </c>
       <c r="H554" t="n">
-        <v>59.5358346770256</v>
+        <v>60.88549117897628</v>
       </c>
       <c r="I554" t="n">
-        <v>4.10244793743407</v>
+        <v>3.876758898677794</v>
       </c>
       <c r="J554" t="n">
-        <v>3.354140974104824</v>
+        <v>2.51635316393893</v>
       </c>
       <c r="K554" t="n">
-        <v>0.1417771050638269</v>
+        <v>0.1140228984790576</v>
       </c>
       <c r="L554" t="n">
-        <v>0.04829969136301014</v>
+        <v>0.04137660131252136</v>
       </c>
     </row>
     <row r="555">
@@ -22626,32 +22626,32 @@
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>CEN01_RP01_0106</t>
+          <t>CEN01_RP01_0107</t>
         </is>
       </c>
       <c r="E555" t="n">
-        <v>171.5431458111511</v>
+        <v>240</v>
       </c>
       <c r="F555" s="2" t="n">
-        <v>45625.56427019872</v>
+        <v>45625.56811260735</v>
       </c>
       <c r="G555" t="n">
-        <v>441458.7632783963</v>
+        <v>384297.2066727304</v>
       </c>
       <c r="H555" t="n">
-        <v>60.88663521942041</v>
+        <v>59.53746955562113</v>
       </c>
       <c r="I555" t="n">
-        <v>3.876534699569179</v>
+        <v>4.102678198007082</v>
       </c>
       <c r="J555" t="n">
-        <v>2.515791112031039</v>
+        <v>3.352948698788143</v>
       </c>
       <c r="K555" t="n">
-        <v>0.1140123324826181</v>
+        <v>0.1417395178397604</v>
       </c>
       <c r="L555" t="n">
-        <v>0.04137485918180678</v>
+        <v>0.04828603087879124</v>
       </c>
     </row>
     <row r="556">
@@ -22673,25 +22673,25 @@
         <v>240</v>
       </c>
       <c r="F556" s="2" t="n">
-        <v>45625.56811260735</v>
+        <v>45625.57245982957</v>
       </c>
       <c r="G556" t="n">
-        <v>384297.2066727304</v>
+        <v>384537.2066727304</v>
       </c>
       <c r="H556" t="n">
-        <v>59.53746955562113</v>
+        <v>59.53910239347337</v>
       </c>
       <c r="I556" t="n">
-        <v>4.102678198007082</v>
+        <v>4.102908171156477</v>
       </c>
       <c r="J556" t="n">
-        <v>3.352948698788143</v>
+        <v>3.351757911733566</v>
       </c>
       <c r="K556" t="n">
-        <v>0.1417395178397604</v>
+        <v>0.1417019775340864</v>
       </c>
       <c r="L556" t="n">
-        <v>0.04828603087879124</v>
+        <v>0.04827238744632263</v>
       </c>
     </row>
     <row r="557">
@@ -22713,25 +22713,25 @@
         <v>240</v>
       </c>
       <c r="F557" s="2" t="n">
-        <v>45625.57245982957</v>
+        <v>45625.5768070518</v>
       </c>
       <c r="G557" t="n">
-        <v>384537.2066727304</v>
+        <v>384777.2066727304</v>
       </c>
       <c r="H557" t="n">
-        <v>59.53910239347337</v>
+        <v>59.54073319440099</v>
       </c>
       <c r="I557" t="n">
-        <v>4.102908171156477</v>
+        <v>4.103137857420085</v>
       </c>
       <c r="J557" t="n">
-        <v>3.351757911733566</v>
+        <v>3.350568610156237</v>
       </c>
       <c r="K557" t="n">
-        <v>0.1417019775340864</v>
+        <v>0.1416644840590104</v>
       </c>
       <c r="L557" t="n">
-        <v>0.04827238744632263</v>
+        <v>0.04825876103369686</v>
       </c>
     </row>
     <row r="558">
@@ -22753,25 +22753,25 @@
         <v>240</v>
       </c>
       <c r="F558" s="2" t="n">
-        <v>45625.5768070518</v>
+        <v>45625.58115427402</v>
       </c>
       <c r="G558" t="n">
-        <v>384777.2066727304</v>
+        <v>385017.2066727304</v>
       </c>
       <c r="H558" t="n">
-        <v>59.54073319440099</v>
+        <v>59.54236196221311</v>
       </c>
       <c r="I558" t="n">
-        <v>4.103137857420085</v>
+        <v>4.103367257334397</v>
       </c>
       <c r="J558" t="n">
-        <v>3.350568610156237</v>
+        <v>3.349380791278245</v>
       </c>
       <c r="K558" t="n">
-        <v>0.1416644840590104</v>
+        <v>0.1416270373269572</v>
       </c>
       <c r="L558" t="n">
-        <v>0.04825876103369686</v>
+        <v>0.04824515160908602</v>
       </c>
     </row>
     <row r="559">
@@ -22793,25 +22793,25 @@
         <v>240</v>
       </c>
       <c r="F559" s="2" t="n">
-        <v>45625.58115427402</v>
+        <v>45625.58550149624</v>
       </c>
       <c r="G559" t="n">
-        <v>385017.2066727304</v>
+        <v>385257.2066727304</v>
       </c>
       <c r="H559" t="n">
-        <v>59.54236196221311</v>
+        <v>59.54398870070941</v>
       </c>
       <c r="I559" t="n">
-        <v>4.103367257334397</v>
+        <v>4.103596371434564</v>
       </c>
       <c r="J559" t="n">
-        <v>3.349380791278245</v>
+        <v>3.348194452328601</v>
       </c>
       <c r="K559" t="n">
-        <v>0.1416270373269572</v>
+        <v>0.1415896372505695</v>
       </c>
       <c r="L559" t="n">
-        <v>0.04824515160908602</v>
+        <v>0.04823155914074155</v>
       </c>
     </row>
     <row r="560">
@@ -22833,25 +22833,25 @@
         <v>240</v>
       </c>
       <c r="F560" s="2" t="n">
-        <v>45625.58550149624</v>
+        <v>45625.58984871846</v>
       </c>
       <c r="G560" t="n">
-        <v>385257.2066727304</v>
+        <v>385497.2066727304</v>
       </c>
       <c r="H560" t="n">
-        <v>59.54398870070941</v>
+        <v>59.54561341368005</v>
       </c>
       <c r="I560" t="n">
-        <v>4.103596371434564</v>
+        <v>4.103825200254407</v>
       </c>
       <c r="J560" t="n">
-        <v>3.348194452328601</v>
+        <v>3.347009590543216</v>
       </c>
       <c r="K560" t="n">
-        <v>0.1415896372505695</v>
+        <v>0.1415522837427077</v>
       </c>
       <c r="L560" t="n">
-        <v>0.04823155914074155</v>
+        <v>0.04821798359699392</v>
       </c>
     </row>
     <row r="561">
@@ -22873,25 +22873,25 @@
         <v>240</v>
       </c>
       <c r="F561" s="2" t="n">
-        <v>45625.58984871846</v>
+        <v>45625.59419594068</v>
       </c>
       <c r="G561" t="n">
-        <v>385497.2066727304</v>
+        <v>385737.2066727304</v>
       </c>
       <c r="H561" t="n">
-        <v>59.54561341368005</v>
+        <v>59.54723610490581</v>
       </c>
       <c r="I561" t="n">
-        <v>4.103825200254407</v>
+        <v>4.104053744326418</v>
       </c>
       <c r="J561" t="n">
-        <v>3.347009590543216</v>
+        <v>3.345826203164882</v>
       </c>
       <c r="K561" t="n">
-        <v>0.1415522837427077</v>
+        <v>0.1415149767164492</v>
       </c>
       <c r="L561" t="n">
-        <v>0.04821798359699392</v>
+        <v>0.04820442494625242</v>
       </c>
     </row>
     <row r="562">
@@ -22913,25 +22913,25 @@
         <v>240</v>
       </c>
       <c r="F562" s="2" t="n">
-        <v>45625.59419594068</v>
+        <v>45625.5985431629</v>
       </c>
       <c r="G562" t="n">
-        <v>385737.2066727304</v>
+        <v>385977.2066727304</v>
       </c>
       <c r="H562" t="n">
-        <v>59.54723610490581</v>
+        <v>59.54885677815803</v>
       </c>
       <c r="I562" t="n">
-        <v>4.104053744326418</v>
+        <v>4.104282004181763</v>
       </c>
       <c r="J562" t="n">
-        <v>3.345826203164882</v>
+        <v>3.344644287443246</v>
       </c>
       <c r="K562" t="n">
-        <v>0.1415149767164492</v>
+        <v>0.1414777160850872</v>
       </c>
       <c r="L562" t="n">
-        <v>0.04820442494625242</v>
+        <v>0.04819088315700493</v>
       </c>
     </row>
     <row r="563">
@@ -22953,25 +22953,25 @@
         <v>240</v>
       </c>
       <c r="F563" s="2" t="n">
-        <v>45625.5985431629</v>
+        <v>45625.60289038513</v>
       </c>
       <c r="G563" t="n">
-        <v>385977.2066727304</v>
+        <v>386217.2066727304</v>
       </c>
       <c r="H563" t="n">
-        <v>59.54885677815803</v>
+        <v>59.5504754371987</v>
       </c>
       <c r="I563" t="n">
-        <v>4.104282004181763</v>
+        <v>4.10450998035029</v>
       </c>
       <c r="J563" t="n">
-        <v>3.344644287443246</v>
+        <v>3.343463840634793</v>
       </c>
       <c r="K563" t="n">
-        <v>0.1414777160850872</v>
+        <v>0.1414405017621309</v>
       </c>
       <c r="L563" t="n">
-        <v>0.04819088315700493</v>
+        <v>0.04817735819781763</v>
       </c>
     </row>
     <row r="564">
@@ -22993,25 +22993,25 @@
         <v>240</v>
       </c>
       <c r="F564" s="2" t="n">
-        <v>45625.60289038513</v>
+        <v>45625.60723760735</v>
       </c>
       <c r="G564" t="n">
-        <v>386217.2066727304</v>
+        <v>386457.2066727304</v>
       </c>
       <c r="H564" t="n">
-        <v>59.5504754371987</v>
+        <v>59.55209208578044</v>
       </c>
       <c r="I564" t="n">
-        <v>4.10450998035029</v>
+        <v>4.104737673360529</v>
       </c>
       <c r="J564" t="n">
-        <v>3.343463840634793</v>
+        <v>3.342284860002823</v>
       </c>
       <c r="K564" t="n">
-        <v>0.1414405017621309</v>
+        <v>0.1414033336613039</v>
       </c>
       <c r="L564" t="n">
-        <v>0.04817735819781763</v>
+        <v>0.04816385003733482</v>
       </c>
     </row>
     <row r="565">
@@ -23033,25 +23033,25 @@
         <v>240</v>
       </c>
       <c r="F565" s="2" t="n">
-        <v>45625.60723760735</v>
+        <v>45625.61158482957</v>
       </c>
       <c r="G565" t="n">
-        <v>386457.2066727304</v>
+        <v>386697.2066727304</v>
       </c>
       <c r="H565" t="n">
-        <v>59.55209208578044</v>
+        <v>59.55370672764658</v>
       </c>
       <c r="I565" t="n">
-        <v>4.104737673360529</v>
+        <v>4.104965083739699</v>
       </c>
       <c r="J565" t="n">
-        <v>3.342284860002823</v>
+        <v>3.341107342817429</v>
       </c>
       <c r="K565" t="n">
-        <v>0.1414033336613039</v>
+        <v>0.1413662116965444</v>
       </c>
       <c r="L565" t="n">
-        <v>0.04816385003733482</v>
+        <v>0.04815035864427861</v>
       </c>
     </row>
     <row r="566">
@@ -23070,28 +23070,28 @@
         </is>
       </c>
       <c r="E566" t="n">
-        <v>240</v>
+        <v>232.3566435834532</v>
       </c>
       <c r="F566" s="2" t="n">
-        <v>45625.61158482957</v>
+        <v>45625.61593205179</v>
       </c>
       <c r="G566" t="n">
-        <v>386697.2066727304</v>
+        <v>386929.5633163138</v>
       </c>
       <c r="H566" t="n">
-        <v>59.55370672764658</v>
+        <v>59.55526803914846</v>
       </c>
       <c r="I566" t="n">
-        <v>4.104965083739699</v>
+        <v>4.105184982931024</v>
       </c>
       <c r="J566" t="n">
-        <v>3.341107342817429</v>
+        <v>3.339968718108282</v>
       </c>
       <c r="K566" t="n">
-        <v>0.1413662116965444</v>
+        <v>0.1413303158413912</v>
       </c>
       <c r="L566" t="n">
-        <v>0.04815035864427861</v>
+        <v>0.04813731286143554</v>
       </c>
     </row>
     <row r="567">
@@ -23110,28 +23110,28 @@
         </is>
       </c>
       <c r="E567" t="n">
-        <v>232.3566435834532</v>
+        <v>240</v>
       </c>
       <c r="F567" s="2" t="n">
-        <v>45625.61593205179</v>
+        <v>45625.70924535386</v>
       </c>
       <c r="G567" t="n">
-        <v>386929.5633163138</v>
+        <v>387169.5633163138</v>
       </c>
       <c r="H567" t="n">
-        <v>59.55526803914846</v>
+        <v>59.55452979948172</v>
       </c>
       <c r="I567" t="n">
-        <v>4.105184982931024</v>
+        <v>4.107123310101342</v>
       </c>
       <c r="J567" t="n">
-        <v>3.339968718108282</v>
+        <v>3.339223126203088</v>
       </c>
       <c r="K567" t="n">
-        <v>0.1413303158413912</v>
+        <v>0.1412956957754771</v>
       </c>
       <c r="L567" t="n">
-        <v>0.04813731286143554</v>
+        <v>0.04813618943870825</v>
       </c>
     </row>
     <row r="568">
@@ -23153,25 +23153,25 @@
         <v>240</v>
       </c>
       <c r="F568" s="2" t="n">
-        <v>45625.70924535386</v>
+        <v>45625.71359257609</v>
       </c>
       <c r="G568" t="n">
-        <v>387169.5633163138</v>
+        <v>387409.5633163138</v>
       </c>
       <c r="H568" t="n">
-        <v>59.55452979948172</v>
+        <v>59.55379247449307</v>
       </c>
       <c r="I568" t="n">
-        <v>4.107123310101342</v>
+        <v>4.109059235686543</v>
       </c>
       <c r="J568" t="n">
-        <v>3.339223126203088</v>
+        <v>3.338478458085401</v>
       </c>
       <c r="K568" t="n">
-        <v>0.1412956957754771</v>
+        <v>0.1412611186037846</v>
       </c>
       <c r="L568" t="n">
-        <v>0.04813618943870825</v>
+        <v>0.04813506740790042</v>
       </c>
     </row>
     <row r="569">
@@ -23193,25 +23193,25 @@
         <v>240</v>
       </c>
       <c r="F569" s="2" t="n">
-        <v>45625.71359257609</v>
+        <v>45625.71793979831</v>
       </c>
       <c r="G569" t="n">
-        <v>387409.5633163138</v>
+        <v>387649.5633163138</v>
       </c>
       <c r="H569" t="n">
-        <v>59.55379247449307</v>
+        <v>59.55305606248363</v>
       </c>
       <c r="I569" t="n">
-        <v>4.109059235686543</v>
+        <v>4.110992764147205</v>
       </c>
       <c r="J569" t="n">
-        <v>3.338478458085401</v>
+        <v>3.337734712039426</v>
       </c>
       <c r="K569" t="n">
-        <v>0.1412611186037846</v>
+        <v>0.1412265842466442</v>
       </c>
       <c r="L569" t="n">
-        <v>0.04813506740790042</v>
+        <v>0.04813394676642676</v>
       </c>
     </row>
     <row r="570">
@@ -23233,25 +23233,25 @@
         <v>240</v>
       </c>
       <c r="F570" s="2" t="n">
-        <v>45625.71793979831</v>
+        <v>45625.72228702053</v>
       </c>
       <c r="G570" t="n">
-        <v>387649.5633163138</v>
+        <v>387889.5633163138</v>
       </c>
       <c r="H570" t="n">
-        <v>59.55305606248363</v>
+        <v>59.55232056175875</v>
       </c>
       <c r="I570" t="n">
-        <v>4.110992764147205</v>
+        <v>4.112923899932866</v>
       </c>
       <c r="J570" t="n">
-        <v>3.337734712039426</v>
+        <v>3.336991886353615</v>
       </c>
       <c r="K570" t="n">
-        <v>0.1412265842466442</v>
+        <v>0.1411920926245835</v>
       </c>
       <c r="L570" t="n">
-        <v>0.04813394676642676</v>
+        <v>0.0481328275117084</v>
       </c>
     </row>
     <row r="571">
@@ -23273,25 +23273,25 @@
         <v>240</v>
       </c>
       <c r="F571" s="2" t="n">
-        <v>45625.72228702053</v>
+        <v>45625.72663424275</v>
       </c>
       <c r="G571" t="n">
-        <v>387889.5633163138</v>
+        <v>388129.5633163138</v>
       </c>
       <c r="H571" t="n">
-        <v>59.55232056175875</v>
+        <v>59.55158597062793</v>
       </c>
       <c r="I571" t="n">
-        <v>4.112923899932866</v>
+        <v>4.11485264748206</v>
       </c>
       <c r="J571" t="n">
-        <v>3.336991886353615</v>
+        <v>3.336249979320653</v>
       </c>
       <c r="K571" t="n">
-        <v>0.1411920926245835</v>
+        <v>0.1411576436583268</v>
       </c>
       <c r="L571" t="n">
-        <v>0.0481328275117084</v>
+        <v>0.04813170964117284</v>
       </c>
     </row>
     <row r="572">
@@ -23313,25 +23313,25 @@
         <v>240</v>
       </c>
       <c r="F572" s="2" t="n">
-        <v>45625.72663424275</v>
+        <v>45625.73098146498</v>
       </c>
       <c r="G572" t="n">
-        <v>388129.5633163138</v>
+        <v>388369.5633163138</v>
       </c>
       <c r="H572" t="n">
-        <v>59.55158597062793</v>
+        <v>59.55085228740487</v>
       </c>
       <c r="I572" t="n">
-        <v>4.11485264748206</v>
+        <v>4.116779011222349</v>
       </c>
       <c r="J572" t="n">
-        <v>3.336249979320653</v>
+        <v>3.335508989237446</v>
       </c>
       <c r="K572" t="n">
-        <v>0.1411576436583268</v>
+        <v>0.1411232372687944</v>
       </c>
       <c r="L572" t="n">
-        <v>0.04813170964117284</v>
+        <v>0.04813059315225393</v>
       </c>
     </row>
     <row r="573">
@@ -23353,25 +23353,25 @@
         <v>240</v>
       </c>
       <c r="F573" s="2" t="n">
-        <v>45625.73098146498</v>
+        <v>45625.7353286872</v>
       </c>
       <c r="G573" t="n">
-        <v>388369.5633163138</v>
+        <v>388609.5633163138</v>
       </c>
       <c r="H573" t="n">
-        <v>59.55085228740487</v>
+        <v>59.55011951040745</v>
       </c>
       <c r="I573" t="n">
-        <v>4.116779011222349</v>
+        <v>4.118702995570356</v>
       </c>
       <c r="J573" t="n">
-        <v>3.335508989237446</v>
+        <v>3.334768914405106</v>
       </c>
       <c r="K573" t="n">
-        <v>0.1411232372687944</v>
+        <v>0.1410888733771018</v>
       </c>
       <c r="L573" t="n">
-        <v>0.04813059315225393</v>
+        <v>0.04812947804239188</v>
       </c>
     </row>
     <row r="574">
@@ -23393,25 +23393,25 @@
         <v>240</v>
       </c>
       <c r="F574" s="2" t="n">
-        <v>45625.7353286872</v>
+        <v>45625.73967590942</v>
       </c>
       <c r="G574" t="n">
-        <v>388609.5633163138</v>
+        <v>388849.5633163138</v>
       </c>
       <c r="H574" t="n">
-        <v>59.55011951040745</v>
+        <v>59.54938763795768</v>
       </c>
       <c r="I574" t="n">
-        <v>4.118702995570356</v>
+        <v>4.120624604931802</v>
       </c>
       <c r="J574" t="n">
-        <v>3.334768914405106</v>
+        <v>3.33402975312894</v>
       </c>
       <c r="K574" t="n">
-        <v>0.1410888733771018</v>
+        <v>0.1410545519045593</v>
       </c>
       <c r="L574" t="n">
-        <v>0.04812947804239188</v>
+        <v>0.04812836430903319</v>
       </c>
     </row>
     <row r="575">
@@ -23433,25 +23433,25 @@
         <v>240</v>
       </c>
       <c r="F575" s="2" t="n">
-        <v>45625.73967590942</v>
+        <v>45625.74402313164</v>
       </c>
       <c r="G575" t="n">
-        <v>388849.5633163138</v>
+        <v>389089.5633163138</v>
       </c>
       <c r="H575" t="n">
-        <v>59.54938763795768</v>
+        <v>59.54865666838172</v>
       </c>
       <c r="I575" t="n">
-        <v>4.120624604931802</v>
+        <v>4.122543843701537</v>
       </c>
       <c r="J575" t="n">
-        <v>3.33402975312894</v>
+        <v>3.333291503718438</v>
       </c>
       <c r="K575" t="n">
-        <v>0.1410545519045593</v>
+        <v>0.1410202727726715</v>
       </c>
       <c r="L575" t="n">
-        <v>0.04812836430903319</v>
+        <v>0.0481272519496307</v>
       </c>
     </row>
     <row r="576">
@@ -23473,25 +23473,25 @@
         <v>240</v>
       </c>
       <c r="F576" s="2" t="n">
-        <v>45625.74402313164</v>
+        <v>45625.74837035387</v>
       </c>
       <c r="G576" t="n">
-        <v>389089.5633163138</v>
+        <v>389329.5633163138</v>
       </c>
       <c r="H576" t="n">
-        <v>59.54865666838172</v>
+        <v>59.54792660000984</v>
       </c>
       <c r="I576" t="n">
-        <v>4.122543843701537</v>
+        <v>4.124460716263576</v>
       </c>
       <c r="J576" t="n">
-        <v>3.333291503718438</v>
+        <v>3.332554164487255</v>
       </c>
       <c r="K576" t="n">
-        <v>0.1410202727726715</v>
+        <v>0.1409860359031364</v>
       </c>
       <c r="L576" t="n">
-        <v>0.0481272519496307</v>
+        <v>0.04812614096164348</v>
       </c>
     </row>
     <row r="577">
@@ -23513,25 +23513,25 @@
         <v>240</v>
       </c>
       <c r="F577" s="2" t="n">
-        <v>45625.74837035387</v>
+        <v>45625.56912898894</v>
       </c>
       <c r="G577" t="n">
-        <v>389329.5633163138</v>
+        <v>389569.5633163138</v>
       </c>
       <c r="H577" t="n">
-        <v>59.54792660000984</v>
+        <v>59.54830045287135</v>
       </c>
       <c r="I577" t="n">
-        <v>4.124460716263576</v>
+        <v>4.12343246403439</v>
       </c>
       <c r="J577" t="n">
-        <v>3.332554164487255</v>
+        <v>3.333139837861173</v>
       </c>
       <c r="K577" t="n">
-        <v>0.1409860359031364</v>
+        <v>0.1410228026137113</v>
       </c>
       <c r="L577" t="n">
-        <v>0.04812614096164348</v>
+        <v>0.04811938695907614</v>
       </c>
     </row>
     <row r="578">
@@ -23553,25 +23553,25 @@
         <v>240</v>
       </c>
       <c r="F578" s="2" t="n">
-        <v>45625.56912898894</v>
+        <v>45625.57402166571</v>
       </c>
       <c r="G578" t="n">
-        <v>389569.5633163138</v>
+        <v>389809.5633163138</v>
       </c>
       <c r="H578" t="n">
-        <v>59.54830045287135</v>
+        <v>59.54867384538146</v>
       </c>
       <c r="I578" t="n">
-        <v>4.12343246403439</v>
+        <v>4.122405477964673</v>
       </c>
       <c r="J578" t="n">
-        <v>3.333139837861173</v>
+        <v>3.33372479005417</v>
       </c>
       <c r="K578" t="n">
-        <v>0.1410228026137113</v>
+        <v>0.1410595240508431</v>
       </c>
       <c r="L578" t="n">
-        <v>0.04811938695907614</v>
+        <v>0.04811264127318837</v>
       </c>
     </row>
     <row r="579">
@@ -23593,25 +23593,25 @@
         <v>240</v>
       </c>
       <c r="F579" s="2" t="n">
-        <v>45625.57402166571</v>
+        <v>45625.57891434249</v>
       </c>
       <c r="G579" t="n">
-        <v>389809.5633163138</v>
+        <v>390049.5633163138</v>
       </c>
       <c r="H579" t="n">
-        <v>59.54867384538146</v>
+        <v>59.54904677838996</v>
       </c>
       <c r="I579" t="n">
-        <v>4.122405477964673</v>
+        <v>4.121379755717197</v>
       </c>
       <c r="J579" t="n">
-        <v>3.33372479005417</v>
+        <v>3.33430902239749</v>
       </c>
       <c r="K579" t="n">
-        <v>0.1410595240508431</v>
+        <v>0.141096200298103</v>
       </c>
       <c r="L579" t="n">
-        <v>0.04811264127318837</v>
+        <v>0.04810590388862826</v>
       </c>
     </row>
     <row r="580">
@@ -23633,25 +23633,25 @@
         <v>240</v>
       </c>
       <c r="F580" s="2" t="n">
-        <v>45625.57891434249</v>
+        <v>45625.58380701926</v>
       </c>
       <c r="G580" t="n">
-        <v>390049.5633163138</v>
+        <v>390289.5633163138</v>
       </c>
       <c r="H580" t="n">
-        <v>59.54904677838996</v>
+        <v>59.54941925274452</v>
       </c>
       <c r="I580" t="n">
-        <v>4.121379755717197</v>
+        <v>4.120355294960484</v>
       </c>
       <c r="J580" t="n">
-        <v>3.33430902239749</v>
+        <v>3.334892536219098</v>
       </c>
       <c r="K580" t="n">
-        <v>0.141096200298103</v>
+        <v>0.1411328314388565</v>
       </c>
       <c r="L580" t="n">
-        <v>0.04810590388862826</v>
+        <v>0.04809917479008164</v>
       </c>
     </row>
     <row r="581">
@@ -23673,25 +23673,25 @@
         <v>240</v>
       </c>
       <c r="F581" s="2" t="n">
-        <v>45625.58380701926</v>
+        <v>45625.58869969603</v>
       </c>
       <c r="G581" t="n">
-        <v>390289.5633163138</v>
+        <v>390529.5633163138</v>
       </c>
       <c r="H581" t="n">
-        <v>59.54941925274452</v>
+        <v>59.54979126929074</v>
       </c>
       <c r="I581" t="n">
-        <v>4.120355294960484</v>
+        <v>4.119332093368786</v>
       </c>
       <c r="J581" t="n">
-        <v>3.334892536219098</v>
+        <v>3.335475332843699</v>
       </c>
       <c r="K581" t="n">
-        <v>0.1411328314388565</v>
+        <v>0.1411694175562642</v>
       </c>
       <c r="L581" t="n">
-        <v>0.04809917479008164</v>
+        <v>0.04809245396227201</v>
       </c>
     </row>
     <row r="582">
@@ -23713,25 +23713,25 @@
         <v>240</v>
       </c>
       <c r="F582" s="2" t="n">
-        <v>45625.58869969603</v>
+        <v>45625.5935923728</v>
       </c>
       <c r="G582" t="n">
-        <v>390529.5633163138</v>
+        <v>390769.5633163138</v>
       </c>
       <c r="H582" t="n">
-        <v>59.54979126929074</v>
+        <v>59.55016282887215</v>
       </c>
       <c r="I582" t="n">
-        <v>4.119332093368786</v>
+        <v>4.118310148622068</v>
       </c>
       <c r="J582" t="n">
-        <v>3.335475332843699</v>
+        <v>3.336057413592739</v>
       </c>
       <c r="K582" t="n">
-        <v>0.1411694175562642</v>
+        <v>0.1412059587332825</v>
       </c>
       <c r="L582" t="n">
-        <v>0.04809245396227201</v>
+        <v>0.04808574138996037</v>
       </c>
     </row>
     <row r="583">
@@ -23753,25 +23753,25 @@
         <v>240</v>
       </c>
       <c r="F583" s="2" t="n">
-        <v>45625.5935923728</v>
+        <v>45625.59848504957</v>
       </c>
       <c r="G583" t="n">
-        <v>390769.5633163138</v>
+        <v>391009.5633163138</v>
       </c>
       <c r="H583" t="n">
-        <v>59.55016282887215</v>
+        <v>59.55053393233019</v>
       </c>
       <c r="I583" t="n">
-        <v>4.118310148622068</v>
+        <v>4.117289458405991</v>
       </c>
       <c r="J583" t="n">
-        <v>3.336057413592739</v>
+        <v>3.336638779784425</v>
       </c>
       <c r="K583" t="n">
-        <v>0.1412059587332825</v>
+        <v>0.141242455052664</v>
       </c>
       <c r="L583" t="n">
-        <v>0.04808574138996037</v>
+        <v>0.04807903705794517</v>
       </c>
     </row>
     <row r="584">
@@ -23793,25 +23793,25 @@
         <v>240</v>
       </c>
       <c r="F584" s="2" t="n">
-        <v>45625.59848504957</v>
+        <v>45625.60337772634</v>
       </c>
       <c r="G584" t="n">
-        <v>391009.5633163138</v>
+        <v>391249.5633163138</v>
       </c>
       <c r="H584" t="n">
-        <v>59.55053393233019</v>
+        <v>59.55092583818333</v>
       </c>
       <c r="I584" t="n">
-        <v>4.117289458405991</v>
+        <v>4.116262714303941</v>
       </c>
       <c r="J584" t="n">
-        <v>3.336638779784425</v>
+        <v>3.337203493758155</v>
       </c>
       <c r="K584" t="n">
-        <v>0.141242455052664</v>
+        <v>0.1412794346732965</v>
       </c>
       <c r="L584" t="n">
-        <v>0.04807903705794517</v>
+        <v>0.04807220742418991</v>
       </c>
     </row>
     <row r="585">
@@ -23833,25 +23833,25 @@
         <v>240</v>
       </c>
       <c r="F585" s="2" t="n">
-        <v>45625.60337772634</v>
+        <v>45625.64093092067</v>
       </c>
       <c r="G585" t="n">
-        <v>391249.5633163138</v>
+        <v>391489.5633163138</v>
       </c>
       <c r="H585" t="n">
-        <v>59.55092583818333</v>
+        <v>59.5518534951961</v>
       </c>
       <c r="I585" t="n">
-        <v>4.116262714303941</v>
+        <v>4.115052930197768</v>
       </c>
       <c r="J585" t="n">
-        <v>3.337203493758155</v>
+        <v>3.337365449650315</v>
       </c>
       <c r="K585" t="n">
-        <v>0.1412794346732965</v>
+        <v>0.1413296898461592</v>
       </c>
       <c r="L585" t="n">
-        <v>0.04807220742418991</v>
+        <v>0.04806201790662522</v>
       </c>
     </row>
     <row r="586">
@@ -23873,25 +23873,25 @@
         <v>240</v>
       </c>
       <c r="F586" s="2" t="n">
-        <v>45625.64093092067</v>
+        <v>45625.64582359744</v>
       </c>
       <c r="G586" t="n">
-        <v>391489.5633163138</v>
+        <v>391729.5633163138</v>
       </c>
       <c r="H586" t="n">
-        <v>59.5518534951961</v>
+        <v>59.55278001551812</v>
       </c>
       <c r="I586" t="n">
-        <v>4.115052930197768</v>
+        <v>4.113844628482574</v>
       </c>
       <c r="J586" t="n">
-        <v>3.337365449650315</v>
+        <v>3.337527207092228</v>
       </c>
       <c r="K586" t="n">
-        <v>0.1413296898461592</v>
+        <v>0.1413798834395925</v>
       </c>
       <c r="L586" t="n">
-        <v>0.04806201790662522</v>
+        <v>0.04805184087463447</v>
       </c>
     </row>
     <row r="587">
@@ -23913,25 +23913,25 @@
         <v>240</v>
       </c>
       <c r="F587" s="2" t="n">
-        <v>45625.64582359744</v>
+        <v>45625.65071627421</v>
       </c>
       <c r="G587" t="n">
-        <v>391729.5633163138</v>
+        <v>391969.5633163138</v>
       </c>
       <c r="H587" t="n">
-        <v>59.55278001551812</v>
+        <v>59.55370540123737</v>
       </c>
       <c r="I587" t="n">
-        <v>4.113844628482574</v>
+        <v>4.112637806435388</v>
       </c>
       <c r="J587" t="n">
-        <v>3.337527207092228</v>
+        <v>3.337688766448424</v>
       </c>
       <c r="K587" t="n">
-        <v>0.1413798834395925</v>
+        <v>0.1414300155667104</v>
       </c>
       <c r="L587" t="n">
-        <v>0.04805184087463447</v>
+        <v>0.04804167630528321</v>
       </c>
     </row>
     <row r="588">
@@ -23953,25 +23953,25 @@
         <v>240</v>
       </c>
       <c r="F588" s="2" t="n">
-        <v>45625.65071627421</v>
+        <v>45625.65560895098</v>
       </c>
       <c r="G588" t="n">
-        <v>391969.5633163138</v>
+        <v>392209.5633163138</v>
       </c>
       <c r="H588" t="n">
-        <v>59.55370540123737</v>
+        <v>59.5546296544367</v>
       </c>
       <c r="I588" t="n">
-        <v>4.112637806435388</v>
+        <v>4.111432461339906</v>
       </c>
       <c r="J588" t="n">
-        <v>3.337688766448424</v>
+        <v>3.337850128082539</v>
       </c>
       <c r="K588" t="n">
-        <v>0.1414300155667104</v>
+        <v>0.1414800863403497</v>
       </c>
       <c r="L588" t="n">
-        <v>0.04804167630528321</v>
+        <v>0.0480315241756931</v>
       </c>
     </row>
     <row r="589">
@@ -23993,25 +23993,25 @@
         <v>240</v>
       </c>
       <c r="F589" s="2" t="n">
-        <v>45625.65560895098</v>
+        <v>45625.66050162775</v>
       </c>
       <c r="G589" t="n">
-        <v>392209.5633163138</v>
+        <v>392449.5633163138</v>
       </c>
       <c r="H589" t="n">
-        <v>59.5546296544367</v>
+        <v>59.55555277719386</v>
       </c>
       <c r="I589" t="n">
-        <v>4.111432461339906</v>
+        <v>4.110228590486467</v>
       </c>
       <c r="J589" t="n">
-        <v>3.337850128082539</v>
+        <v>3.33801129235732</v>
       </c>
       <c r="K589" t="n">
-        <v>0.1414800863403497</v>
+        <v>0.1415300958730715</v>
       </c>
       <c r="L589" t="n">
-        <v>0.0480315241756931</v>
+        <v>0.04802138446304177</v>
       </c>
     </row>
     <row r="590">
@@ -24033,25 +24033,25 @@
         <v>240</v>
       </c>
       <c r="F590" s="2" t="n">
-        <v>45625.66050162775</v>
+        <v>45625.66539430452</v>
       </c>
       <c r="G590" t="n">
-        <v>392449.5633163138</v>
+        <v>392689.5633163138</v>
       </c>
       <c r="H590" t="n">
-        <v>59.55555277719386</v>
+        <v>59.55647477158153</v>
       </c>
       <c r="I590" t="n">
-        <v>4.110228590486467</v>
+        <v>4.109026191172034</v>
       </c>
       <c r="J590" t="n">
-        <v>3.33801129235732</v>
+        <v>3.338172259634628</v>
       </c>
       <c r="K590" t="n">
-        <v>0.1415300958730715</v>
+        <v>0.1415800442771615</v>
       </c>
       <c r="L590" t="n">
-        <v>0.04802138446304177</v>
+        <v>0.04801125714456266</v>
       </c>
     </row>
     <row r="591">
@@ -24073,25 +24073,25 @@
         <v>240</v>
       </c>
       <c r="F591" s="2" t="n">
-        <v>45625.66539430452</v>
+        <v>45625.67028698129</v>
       </c>
       <c r="G591" t="n">
-        <v>392689.5633163138</v>
+        <v>392929.5633163138</v>
       </c>
       <c r="H591" t="n">
-        <v>59.55647477158153</v>
+        <v>59.55739563966731</v>
       </c>
       <c r="I591" t="n">
-        <v>4.109026191172034</v>
+        <v>4.107825260700174</v>
       </c>
       <c r="J591" t="n">
-        <v>3.338172259634628</v>
+        <v>3.338333030275438</v>
       </c>
       <c r="K591" t="n">
-        <v>0.1415800442771615</v>
+        <v>0.1416299316646313</v>
       </c>
       <c r="L591" t="n">
-        <v>0.04801125714456266</v>
+        <v>0.0480011421975448</v>
       </c>
     </row>
     <row r="592">
@@ -24113,25 +24113,25 @@
         <v>240</v>
       </c>
       <c r="F592" s="2" t="n">
-        <v>45625.67028698129</v>
+        <v>45625.67517965806</v>
       </c>
       <c r="G592" t="n">
-        <v>392929.5633163138</v>
+        <v>393169.5633163138</v>
       </c>
       <c r="H592" t="n">
-        <v>59.55739563966731</v>
+        <v>59.55831538351378</v>
       </c>
       <c r="I592" t="n">
-        <v>4.107825260700174</v>
+        <v>4.106625796381039</v>
       </c>
       <c r="J592" t="n">
-        <v>3.338333030275438</v>
+        <v>3.338493604639845</v>
       </c>
       <c r="K592" t="n">
-        <v>0.1416299316646313</v>
+        <v>0.1416797581472187</v>
       </c>
       <c r="L592" t="n">
-        <v>0.0480011421975448</v>
+        <v>0.0479910395993327</v>
       </c>
     </row>
     <row r="593">
@@ -24153,25 +24153,25 @@
         <v>240</v>
       </c>
       <c r="F593" s="2" t="n">
-        <v>45625.67517965806</v>
+        <v>45625.68007233484</v>
       </c>
       <c r="G593" t="n">
-        <v>393169.5633163138</v>
+        <v>393409.5633163138</v>
       </c>
       <c r="H593" t="n">
-        <v>59.55831538351378</v>
+        <v>59.55923400517846</v>
       </c>
       <c r="I593" t="n">
-        <v>4.106625796381039</v>
+        <v>4.105427795531343</v>
       </c>
       <c r="J593" t="n">
-        <v>3.338493604639845</v>
+        <v>3.338653983087065</v>
       </c>
       <c r="K593" t="n">
-        <v>0.1416797581472187</v>
+        <v>0.1417295238363891</v>
       </c>
       <c r="L593" t="n">
-        <v>0.0479910395993327</v>
+        <v>0.04798094932732615</v>
       </c>
     </row>
     <row r="594">
@@ -24193,25 +24193,25 @@
         <v>240</v>
       </c>
       <c r="F594" s="2" t="n">
-        <v>45625.68007233484</v>
+        <v>45625.68496501161</v>
       </c>
       <c r="G594" t="n">
-        <v>393409.5633163138</v>
+        <v>393649.5633163138</v>
       </c>
       <c r="H594" t="n">
-        <v>59.55923400517846</v>
+        <v>59.56015150671387</v>
       </c>
       <c r="I594" t="n">
-        <v>4.105427795531343</v>
+        <v>4.104231255474346</v>
       </c>
       <c r="J594" t="n">
-        <v>3.338653983087065</v>
+        <v>3.338814165975439</v>
       </c>
       <c r="K594" t="n">
-        <v>0.1417295238363891</v>
+        <v>0.141779228843336</v>
       </c>
       <c r="L594" t="n">
-        <v>0.04798094932732615</v>
+        <v>0.04797087135898005</v>
       </c>
     </row>
     <row r="595">
@@ -24233,25 +24233,25 @@
         <v>240</v>
       </c>
       <c r="F595" s="2" t="n">
-        <v>45625.68496501161</v>
+        <v>45625.68985768838</v>
       </c>
       <c r="G595" t="n">
-        <v>393649.5633163138</v>
+        <v>393889.5633163138</v>
       </c>
       <c r="H595" t="n">
-        <v>59.56015150671387</v>
+        <v>59.56106789016751</v>
       </c>
       <c r="I595" t="n">
-        <v>4.104231255474346</v>
+        <v>4.10303617353983</v>
       </c>
       <c r="J595" t="n">
-        <v>3.338814165975439</v>
+        <v>3.338974153662432</v>
       </c>
       <c r="K595" t="n">
-        <v>0.141779228843336</v>
+        <v>0.1418288732789818</v>
       </c>
       <c r="L595" t="n">
-        <v>0.04797087135898005</v>
+        <v>0.04796080567180425</v>
       </c>
     </row>
     <row r="596">
@@ -24273,25 +24273,25 @@
         <v>240</v>
       </c>
       <c r="F596" s="2" t="n">
-        <v>45625.68985768838</v>
+        <v>45625.69475036515</v>
       </c>
       <c r="G596" t="n">
-        <v>393889.5633163138</v>
+        <v>394129.5633163138</v>
       </c>
       <c r="H596" t="n">
-        <v>59.56106789016751</v>
+        <v>59.56198315758193</v>
       </c>
       <c r="I596" t="n">
-        <v>4.10303617353983</v>
+        <v>4.101842547064082</v>
       </c>
       <c r="J596" t="n">
-        <v>3.338974153662432</v>
+        <v>3.339133946504641</v>
       </c>
       <c r="K596" t="n">
-        <v>0.1418288732789818</v>
+        <v>0.1418784572539788</v>
       </c>
       <c r="L596" t="n">
-        <v>0.04796080567180425</v>
+        <v>0.04795075224336338</v>
       </c>
     </row>
     <row r="597">
@@ -24313,25 +24313,25 @@
         <v>240</v>
       </c>
       <c r="F597" s="2" t="n">
-        <v>45625.69475036515</v>
+        <v>45625.69964304192</v>
       </c>
       <c r="G597" t="n">
-        <v>394129.5633163138</v>
+        <v>394369.5633163138</v>
       </c>
       <c r="H597" t="n">
-        <v>59.56198315758193</v>
+        <v>59.56289731099464</v>
       </c>
       <c r="I597" t="n">
-        <v>4.101842547064082</v>
+        <v>4.100650373389872</v>
       </c>
       <c r="J597" t="n">
-        <v>3.339133946504641</v>
+        <v>3.339293544857794</v>
       </c>
       <c r="K597" t="n">
-        <v>0.1418784572539788</v>
+        <v>0.1419279808787099</v>
       </c>
       <c r="L597" t="n">
-        <v>0.04795075224336338</v>
+        <v>0.04794071105127667</v>
       </c>
     </row>
     <row r="598">
@@ -24353,25 +24353,25 @@
         <v>240</v>
       </c>
       <c r="F598" s="2" t="n">
-        <v>45625.69964304192</v>
+        <v>45625.70453571869</v>
       </c>
       <c r="G598" t="n">
-        <v>394369.5633163138</v>
+        <v>394609.5633163138</v>
       </c>
       <c r="H598" t="n">
-        <v>59.56289731099464</v>
+        <v>59.56381035243827</v>
       </c>
       <c r="I598" t="n">
-        <v>4.100650373389872</v>
+        <v>4.099459649866436</v>
       </c>
       <c r="J598" t="n">
-        <v>3.339293544857794</v>
+        <v>3.339452949076752</v>
       </c>
       <c r="K598" t="n">
-        <v>0.1419279808787099</v>
+        <v>0.1419774442632895</v>
       </c>
       <c r="L598" t="n">
-        <v>0.04794071105127667</v>
+        <v>0.04793068207321784</v>
       </c>
     </row>
     <row r="599">
@@ -24393,25 +24393,25 @@
         <v>240</v>
       </c>
       <c r="F599" s="2" t="n">
-        <v>45625.70453571869</v>
+        <v>45625.70942839546</v>
       </c>
       <c r="G599" t="n">
-        <v>394609.5633163138</v>
+        <v>394849.5633163138</v>
       </c>
       <c r="H599" t="n">
-        <v>59.56381035243827</v>
+        <v>59.56472228394046</v>
       </c>
       <c r="I599" t="n">
-        <v>4.099459649866436</v>
+        <v>4.098270373849454</v>
       </c>
       <c r="J599" t="n">
-        <v>3.339452949076752</v>
+        <v>3.339612159515516</v>
       </c>
       <c r="K599" t="n">
-        <v>0.1419774442632895</v>
+        <v>0.1420268475175643</v>
       </c>
       <c r="L599" t="n">
-        <v>0.04793068207321784</v>
+        <v>0.04792066528691484</v>
       </c>
     </row>
     <row r="600">
@@ -24433,25 +24433,25 @@
         <v>240</v>
       </c>
       <c r="F600" s="2" t="n">
-        <v>45625.70942839546</v>
+        <v>45625.71432107224</v>
       </c>
       <c r="G600" t="n">
-        <v>394849.5633163138</v>
+        <v>395089.5633163138</v>
       </c>
       <c r="H600" t="n">
-        <v>59.56472228394046</v>
+        <v>59.56563310752394</v>
       </c>
       <c r="I600" t="n">
-        <v>4.098270373849454</v>
+        <v>4.097082542701031</v>
       </c>
       <c r="J600" t="n">
-        <v>3.339612159515516</v>
+        <v>3.339771176527226</v>
       </c>
       <c r="K600" t="n">
-        <v>0.1420268475175643</v>
+        <v>0.1420761907511141</v>
       </c>
       <c r="L600" t="n">
-        <v>0.04792066528691484</v>
+        <v>0.04791066067014976</v>
       </c>
     </row>
     <row r="601">
@@ -24473,25 +24473,25 @@
         <v>240</v>
       </c>
       <c r="F601" s="2" t="n">
-        <v>45625.71432107224</v>
+        <v>45625.71921374901</v>
       </c>
       <c r="G601" t="n">
-        <v>395089.5633163138</v>
+        <v>395329.5633163138</v>
       </c>
       <c r="H601" t="n">
-        <v>59.56563310752394</v>
+        <v>59.56654282520651</v>
       </c>
       <c r="I601" t="n">
-        <v>4.097082542701031</v>
+        <v>4.095896153789679</v>
       </c>
       <c r="J601" t="n">
-        <v>3.339771176527226</v>
+        <v>3.339930000464162</v>
       </c>
       <c r="K601" t="n">
-        <v>0.1420761907511141</v>
+        <v>0.1421254740732524</v>
       </c>
       <c r="L601" t="n">
-        <v>0.04791066067014976</v>
+        <v>0.04790066820075867</v>
       </c>
     </row>
     <row r="602">
@@ -24513,25 +24513,25 @@
         <v>240</v>
       </c>
       <c r="F602" s="2" t="n">
-        <v>45625.71921374901</v>
+        <v>45625.72410642578</v>
       </c>
       <c r="G602" t="n">
-        <v>395329.5633163138</v>
+        <v>395569.5633163138</v>
       </c>
       <c r="H602" t="n">
-        <v>59.56654282520651</v>
+        <v>59.5674514390011</v>
       </c>
       <c r="I602" t="n">
-        <v>4.095896153789679</v>
+        <v>4.094711204490294</v>
       </c>
       <c r="J602" t="n">
-        <v>3.339930000464162</v>
+        <v>3.340088631677753</v>
       </c>
       <c r="K602" t="n">
-        <v>0.1421254740732524</v>
+        <v>0.1421746975930277</v>
       </c>
       <c r="L602" t="n">
-        <v>0.04790066820075867</v>
+        <v>0.04789068785663136</v>
       </c>
     </row>
     <row r="603">
@@ -24553,25 +24553,25 @@
         <v>240</v>
       </c>
       <c r="F603" s="2" t="n">
-        <v>45625.72410642578</v>
+        <v>45625.72899910255</v>
       </c>
       <c r="G603" t="n">
-        <v>395569.5633163138</v>
+        <v>395809.5633163138</v>
       </c>
       <c r="H603" t="n">
-        <v>59.5674514390011</v>
+        <v>59.56835895091574</v>
       </c>
       <c r="I603" t="n">
-        <v>4.094711204490294</v>
+        <v>4.093527692184142</v>
       </c>
       <c r="J603" t="n">
-        <v>3.340088631677753</v>
+        <v>3.340247070518573</v>
       </c>
       <c r="K603" t="n">
-        <v>0.1421746975930277</v>
+        <v>0.1422238614192239</v>
       </c>
       <c r="L603" t="n">
-        <v>0.04789068785663136</v>
+        <v>0.04788071961571133</v>
       </c>
     </row>
     <row r="604">
@@ -24593,25 +24593,25 @@
         <v>240</v>
       </c>
       <c r="F604" s="2" t="n">
-        <v>45625.72899910255</v>
+        <v>45625.73389177932</v>
       </c>
       <c r="G604" t="n">
-        <v>395809.5633163138</v>
+        <v>396049.5633163138</v>
       </c>
       <c r="H604" t="n">
-        <v>59.56835895091574</v>
+        <v>59.5692653629536</v>
       </c>
       <c r="I604" t="n">
-        <v>4.093527692184142</v>
+        <v>4.092345614258834</v>
       </c>
       <c r="J604" t="n">
-        <v>3.340247070518573</v>
+        <v>3.340405317336347</v>
       </c>
       <c r="K604" t="n">
-        <v>0.1422238614192239</v>
+        <v>0.1422729656603612</v>
       </c>
       <c r="L604" t="n">
-        <v>0.04788071961571133</v>
+        <v>0.04787076345599547</v>
       </c>
     </row>
     <row r="605">
@@ -24633,25 +24633,25 @@
         <v>240</v>
       </c>
       <c r="F605" s="2" t="n">
-        <v>45625.73389177932</v>
+        <v>45625.73878445609</v>
       </c>
       <c r="G605" t="n">
-        <v>396049.5633163138</v>
+        <v>396289.5633163138</v>
       </c>
       <c r="H605" t="n">
-        <v>59.5692653629536</v>
+        <v>59.57017067711299</v>
       </c>
       <c r="I605" t="n">
-        <v>4.092345614258834</v>
+        <v>4.09116496810831</v>
       </c>
       <c r="J605" t="n">
-        <v>3.340405317336347</v>
+        <v>3.340563372479952</v>
       </c>
       <c r="K605" t="n">
-        <v>0.1422729656603612</v>
+        <v>0.1423220104246968</v>
       </c>
       <c r="L605" t="n">
-        <v>0.04787076345599547</v>
+        <v>0.04786081935553403</v>
       </c>
     </row>
     <row r="606">
@@ -24673,25 +24673,25 @@
         <v>240</v>
       </c>
       <c r="F606" s="2" t="n">
-        <v>45625.73878445609</v>
+        <v>45625.74367713286</v>
       </c>
       <c r="G606" t="n">
-        <v>396289.5633163138</v>
+        <v>396529.5633163138</v>
       </c>
       <c r="H606" t="n">
-        <v>59.57017067711299</v>
+        <v>59.5710748953874</v>
       </c>
       <c r="I606" t="n">
-        <v>4.09116496810831</v>
+        <v>4.08998575113282</v>
       </c>
       <c r="J606" t="n">
-        <v>3.340563372479952</v>
+        <v>3.340721236297421</v>
       </c>
       <c r="K606" t="n">
-        <v>0.1423220104246968</v>
+        <v>0.1423709958202261</v>
       </c>
       <c r="L606" t="n">
-        <v>0.04786081935553403</v>
+        <v>0.04785088729243037</v>
       </c>
     </row>
     <row r="607">
@@ -24713,64 +24713,24 @@
         <v>240</v>
       </c>
       <c r="F607" s="2" t="n">
-        <v>45625.74367713286</v>
+        <v>45625.74856980963</v>
       </c>
       <c r="G607" t="n">
-        <v>396529.5633163138</v>
+        <v>396769.5633163138</v>
       </c>
       <c r="H607" t="n">
-        <v>59.5710748953874</v>
+        <v>59.57197801976546</v>
       </c>
       <c r="I607" t="n">
-        <v>4.08998575113282</v>
+        <v>4.088807960738905</v>
       </c>
       <c r="J607" t="n">
-        <v>3.340721236297421</v>
+        <v>3.340878909135947</v>
       </c>
       <c r="K607" t="n">
-        <v>0.1423709958202261</v>
+        <v>0.1424199219546828</v>
       </c>
       <c r="L607" t="n">
-        <v>0.04785088729243037</v>
-      </c>
-    </row>
-    <row r="608">
-      <c r="A608" t="n">
-        <v>3</v>
-      </c>
-      <c r="B608" s="2" t="n">
-        <v>45625.56427019872</v>
-      </c>
-      <c r="C608" s="2" t="n">
-        <v>45625.75</v>
-      </c>
-      <c r="D608" t="inlineStr">
-        <is>
-          <t>CEN01_RP01_0107</t>
-        </is>
-      </c>
-      <c r="E608" t="n">
-        <v>240</v>
-      </c>
-      <c r="F608" s="2" t="n">
-        <v>45625.74856980963</v>
-      </c>
-      <c r="G608" t="n">
-        <v>396769.5633163138</v>
-      </c>
-      <c r="H608" t="n">
-        <v>59.57197801976546</v>
-      </c>
-      <c r="I608" t="n">
-        <v>4.088807960738905</v>
-      </c>
-      <c r="J608" t="n">
-        <v>3.340878909135947</v>
-      </c>
-      <c r="K608" t="n">
-        <v>0.1424199219546828</v>
-      </c>
-      <c r="L608" t="n">
         <v>0.04784096724484081</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Restructured for Flask app setup
</commit_message>
<xml_diff>
--- a/blendmaster_backend_OOP/output/build_report_2024-11-28_06-00.xlsx
+++ b/blendmaster_backend_OOP/output/build_report_2024-11-28_06-00.xlsx
@@ -30913,22 +30913,22 @@
         <v>45625.56427019872</v>
       </c>
       <c r="J575" t="n">
-        <v>445744.7353634185</v>
+        <v>441287.2201325851</v>
       </c>
       <c r="K575" t="n">
-        <v>60.88547961380101</v>
+        <v>60.88549117897628</v>
       </c>
       <c r="L575" t="n">
-        <v>3.876761165120385</v>
+        <v>3.876758898677794</v>
       </c>
       <c r="M575" t="n">
-        <v>2.516358845756266</v>
+        <v>2.51635316393893</v>
       </c>
       <c r="N575" t="n">
-        <v>0.114023005291366</v>
+        <v>0.1140228984790576</v>
       </c>
       <c r="O575" t="n">
-        <v>0.041376618923828</v>
+        <v>0.04137660131252136</v>
       </c>
     </row>
     <row r="576">

</xml_diff>